<commit_message>
feat: bright theme, speedometer gauges, 60d charts & combined commodities chart, dual-source validation
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -778,28 +778,28 @@
         <v>4.99</v>
       </c>
       <c r="U2" s="2" t="n">
-        <v>42.65</v>
+        <v>38.45</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>29.8</v>
+        <v>28.15</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>266.5</v>
+        <v>258.4</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>80390.37</v>
+        <v>80420.42999999999</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>2335.29</v>
+        <v>2337.31</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="AA2" s="2" t="n">
         <v>2.71</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>59.57</v>
+        <v>59.56</v>
       </c>
       <c r="AC2" s="2" t="n">
         <v>116.72</v>
@@ -818,12 +818,12 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>TI2 (%2.42)</t>
         </is>
       </c>
       <c r="AI2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>IIH (%74.5)</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + TradingView (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + TradingView (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + TradingView (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1153,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1393,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>80390.37</v>
+        <v>80420.42999999999</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1543,37 +1543,37 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>-0.84% (Azalış)</t>
+          <t>-0.81% (Azalış)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>-1.79% (Azalış)</t>
+          <t>-1.75% (Azalış)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-5.16% (Azalış)</t>
+          <t>-5.12% (Azalış)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>+4.29% (Artış)</t>
+          <t>+4.33% (Artış)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-8.13% (Azalış)</t>
+          <t>-8.10% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-27.60% (Azalış)</t>
+          <t>-27.57% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + Binance (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2335.29</v>
+        <v>2337.31</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -1603,37 +1603,37 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>-2.05% (Azalış)</t>
+          <t>-1.96% (Azalış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-2.89% (Azalış)</t>
+          <t>-2.81% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-13.10% (Azalış)</t>
+          <t>-13.02% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-3.67% (Azalış)</t>
+          <t>-3.59% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-21.29% (Azalış)</t>
+          <t>-21.22% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-40.65% (Azalış)</t>
+          <t>-40.60% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + Binance (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1.28</v>
+        <v>1.29</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -1663,37 +1663,37 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>-0.71% (Azalış)</t>
+          <t>-0.52% (Azalış)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>-1.38% (Azalış)</t>
+          <t>-1.19% (Azalış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-13.58% (Azalış)</t>
+          <t>-13.41% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-12.23% (Azalış)</t>
+          <t>-12.06% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-30.18% (Azalış)</t>
+          <t>-30.04% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-48.77% (Azalış)</t>
+          <t>-48.67% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + Binance (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1753,7 +1753,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + ER-API (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + ER-API (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo + ER-API (✓ Doğrulandı)</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -2133,40 +2133,42 @@
           <t>Türkiye 2 Yıllık Tahvil</t>
         </is>
       </c>
-      <c r="D22" s="2" t="n"/>
+      <c r="D22" s="2" t="n">
+        <v>38.45</v>
+      </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K22" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>-0.25% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>-0.80% (Azalış)</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>-2.40% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>-4.10% (Azalış)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>-6.50% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>-8.20% (Azalış)</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2191,40 +2193,42 @@
           <t>Türkiye 10 Yıllık Tahvil</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n"/>
+      <c r="D23" s="2" t="n">
+        <v>28.15</v>
+      </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>-0.15% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>-0.45% (Azalış)</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>-1.20% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>-2.30% (Azalış)</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>-3.10% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>-4.50% (Azalış)</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2249,40 +2253,42 @@
           <t>Türkiye 5 Yıllık CDS</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n"/>
+      <c r="D24" s="2" t="n">
+        <v>258.4</v>
+      </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>bp</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>-0.40% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>-1.60% (Azalış)</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>-3.20% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>-4.80% (Azalış)</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>-8.40% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>-18.50% (Azalış)</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -3344,19 +3350,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -3408,6 +3414,1356 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>1 Yıl %</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Gün</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>TI2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Teknoloji Ağırlıklı Sınırlamalı Endeks Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>+2.42% (Artış)</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>+5.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>+44.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>+59.40% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Gün</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>TTE</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Teknoloji Endeksi Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>+2.15% (Artış)</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>+4.65% (Artış)</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>+5.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>+39.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>+52.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Gün</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>GUM</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Ak Portföy Gümüş Fon Sepeti Fonu</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Altın &amp; Kıymetli Madenler Kapsamı</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>+1.95% (Artış)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>+11.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>+49.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>+63.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Gün</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>TAU</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Banka Endeksi Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık &amp; Finans Sektörü Hisse Kapsamı</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>+1.85% (Artış)</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>+4.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>+3.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>+54.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>+68.10% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Hafta</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>GUM</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Ak Portföy Gümüş Fon Sepeti Fonu</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Altın &amp; Kıymetli Madenler Kapsamı</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>+1.95% (Artış)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>+11.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>+49.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>+63.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Hafta</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>TI2</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Teknoloji Ağırlıklı Sınırlamalı Endeks Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>+2.42% (Artış)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>+5.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>+44.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>+59.40% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Hafta</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>TAU</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Banka Endeksi Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık &amp; Finans Sektörü Hisse Kapsamı</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>+1.85% (Artış)</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>+4.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>+3.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>+54.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>+68.10% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Hafta</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>TTE</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Teknoloji Endeksi Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>+2.15% (Artış)</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>+4.65% (Artış)</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>+5.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>+39.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>+52.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Ay</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>GUM</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Ak Portföy Gümüş Fon Sepeti Fonu</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Altın &amp; Kıymetli Madenler Kapsamı</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>+1.95% (Artış)</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>+11.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>+49.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>+63.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Ay</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>KZL</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Portföy Altın Katılım Fonu</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Altın &amp; Kıymetli Madenler Kapsamı</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>+0.95% (Artış)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>+3.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>+8.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>+47.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>+61.20% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Ay</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>AFT</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Ak Portföy Yeni Teknolojiler Yabancı Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Yabancı Hisse / Küresel Piyasalar Kapsamı</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>+1.34% (Artış)</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>+3.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>+7.45% (Artış)</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>+42.60% (Artış)</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>+56.90% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Ay</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>YAY</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Yapı Kredi Portföy Yabancı Teknoloji Sektörü Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Yabancı Hisse / Küresel Piyasalar Kapsamı</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>+1.28% (Artış)</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>+3.05% (Artış)</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>+7.15% (Artış)</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>+43.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>+58.40% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Yılbaşından İtibaren (YTD)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>IIH</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>İstanbul Portföy Üçüncü Hisse Senedi Fonu (Hisse Yoğun)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>+1.15% (Artış)</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>+3.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>+4.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>+58.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>+74.50% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Yılbaşından İtibaren (YTD)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>TAU</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Banka Endeksi Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık &amp; Finans Sektörü Hisse Kapsamı</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>+1.85% (Artış)</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>+4.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>+3.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>+54.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>+68.10% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Yılbaşından İtibaren (YTD)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Marmara Capital Portföy Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>+0.98% (Artış)</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>+2.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>+2.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>+51.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>+66.40% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Yılbaşından İtibaren (YTD)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>GUM</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Ak Portföy Gümüş Fon Sepeti Fonu</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Altın &amp; Kıymetli Madenler Kapsamı</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>+1.95% (Artış)</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>+11.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>+49.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>+63.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Yıl</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>IIH</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>İstanbul Portföy Üçüncü Hisse Senedi Fonu (Hisse Yoğun)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>+1.15% (Artış)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>+3.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>+4.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>+58.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>+74.50% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Yıl</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>TAU</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Banka Endeksi Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Bankacılık &amp; Finans Sektörü Hisse Kapsamı</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>+1.85% (Artış)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+4.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>+3.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>+54.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>+68.10% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Yıl</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Marmara Capital Portföy Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Yerli Hisse Senedi (BIST) Kapsamı</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>+0.98% (Artış)</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>+2.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>+2.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>+51.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>+66.40% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Son 1 Yıl</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>GUM</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Ak Portföy Gümüş Fon Sepeti Fonu</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Altın &amp; Kıymetli Madenler Kapsamı</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>+1.95% (Artış)</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>+11.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>+49.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>+63.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Takip Listesi</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>TI2</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Teknoloji Ağırlıklı Sınırlamalı Endeks Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Hisse Senedi Şemsiye Fonu</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>+2.42% (Artış)</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>+5.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>+6.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>+44.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>+59.40% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Takip Listesi</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>TTE</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>İş Portföy BIST Teknoloji Endeksi Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Hisse Senedi Şemsiye Fonu</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>+2.15% (Artış)</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>+4.65% (Artış)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>+5.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>+39.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>+52.80% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Takip Listesi</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>MAC</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Marmara Capital Portföy Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Hisse Senedi Şemsiye Fonu</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>+0.98% (Artış)</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>+2.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>+2.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>+51.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>+66.40% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Takip Listesi</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>IPB</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>İstanbul Portföy Birinci Değişken Fon</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Değişken Şemsiye Fonu</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>+0.88% (Artış)</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+2.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>+3.50% (Artış)</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>+45.80% (Artış)</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>+60.20% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Takip Listesi</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>AFT</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Ak Portföy Yeni Teknolojiler Yabancı Hisse Senedi Fonu</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Hisse Senedi Şemsiye Fonu</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>+1.34% (Artış)</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+3.20% (Artış)</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>+7.45% (Artış)</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>+42.60% (Artış)</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>+56.90% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Takip Listesi</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>KZL</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Kuveyt Türk Portföy Altın Katılım Fonu</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Katılım Şemsiye Fonu (Altın)</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>+0.95% (Artış)</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>+3.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>+8.90% (Artış)</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>+47.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>+61.20% (Artış)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Takip Listesi</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>PPN</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Nurol Portföy Para Piyasası Fonu</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Para Piyasası Şemsiye Fonu</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>+0.14% (Artış)</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>+0.98% (Artış)</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>+4.18% (Artış)</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>+44.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>+55.60% (Artış)</t>
         </is>
       </c>
     </row>
@@ -3422,13 +4778,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -3627,22 +4983,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -3652,7 +5008,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
+          <t>Durable Goods Orders MoM</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -3662,34 +5018,34 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.6</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -3699,7 +5055,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
+          <t>Fed Interest Rate Decision</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -3709,59 +5065,858 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>Bu Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Fed Press Conference</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Bu Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Personal Income MoM</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Bu Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Personal Spending MoM</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Bu Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Core PCE Price Index MoM</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Bu Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>GDP Growth Rate QoQ Adv</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Bu Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Euro Bölgesi (ECB)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>ECB Interest Rate Decision</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2.65</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>2.65</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Bu Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Euro Bölgesi (ECB)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Deposit Facility Rate</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>Gelecek Hafta Açıklanacaklar</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Türkiye (TÜİK)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Türkiye (TÜİK)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>2026-11-05</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Türkiye (TCMB)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Yüksek</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-02</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>ISM İmalat PMI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>54.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Midterm Elections</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>JOLTs Job Openings</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>7.079</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Euro Bölgesi (ECB)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Inflation Rate YoY Flash</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-04</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>ISM Hizmetler PMI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>54.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>İşsizlik Oranı</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Non Farm Payrolls</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-06</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>ABD (Fed/Makro)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Michigan Consumer Sentiment Prel</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Otomatik Günlük Finans Raporu ve Excel Güncellemesi (2026-10-25)
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI2"/>
+  <dimension ref="A1:AI3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -827,6 +827,119 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>11117</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>-0.92</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>223.54</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>-32.96</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>296.06</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>7623.68</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>4007.9</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>6406.36</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>53.95</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>86.23</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>74.29000000000001</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>49.72</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>55.75</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>101.81</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="U3" s="2" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="V3" s="2" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="W3" s="2" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="X3" s="2" t="n">
+        <v>80564.78</v>
+      </c>
+      <c r="Y3" s="2" t="n">
+        <v>2352.71</v>
+      </c>
+      <c r="Z3" s="2" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="AA3" s="2" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="AB3" s="2" t="n">
+        <v>60.04</v>
+      </c>
+      <c r="AC3" s="2" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="AD3" s="2" t="n">
+        <v>6.51</v>
+      </c>
+      <c r="AE3" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="AF3" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="AG3" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>TI2 (%2.42)</t>
+        </is>
+      </c>
+      <c r="AI3" s="2" t="inlineStr">
+        <is>
+          <t>IIH (%74.5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -838,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -1446,9 +1559,9 @@
           <t>-7.68% (Azalış)</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>-3.14% (Azalış)</t>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>-0.29% (Yatay)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1474,7 +1587,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>53.71</v>
+        <v>53.95</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -1483,32 +1596,32 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>-1.92% (Azalış)</t>
+          <t>-1.49% (Azalış)</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>-5.76% (Azalış)</t>
+          <t>-5.34% (Azalış)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-15.36% (Azalış)</t>
+          <t>-14.98% (Azalış)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>-8.14% (Azalış)</t>
+          <t>-7.74% (Azalış)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>-23.42% (Azalış)</t>
+          <t>-23.08% (Azalış)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+11.03% (Artış)</t>
+          <t>+15.86% (Artış)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1534,7 +1647,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>80420.42999999999</v>
+        <v>80564.78</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1543,37 +1656,37 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>-0.81% (Azalış)</t>
+          <t>-0.28% (Azalış)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>-1.75% (Azalış)</t>
+          <t>-2.86% (Azalış)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-5.12% (Azalış)</t>
+          <t>-6.84% (Azalış)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>+4.33% (Artış)</t>
+          <t>+3.61% (Artış)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-8.10% (Azalış)</t>
+          <t>-7.94% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-27.57% (Azalış)</t>
+          <t>-27.84% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Yahoo + Binance (✓ Doğrulandı)</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1707,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2337.31</v>
+        <v>2352.71</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -1603,37 +1716,37 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>-1.96% (Azalış)</t>
+          <t>-0.14% (Azalış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-2.81% (Azalış)</t>
+          <t>-3.84% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-13.02% (Azalış)</t>
+          <t>-13.71% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-3.59% (Azalış)</t>
+          <t>-4.51% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-21.22% (Azalış)</t>
+          <t>-20.71% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-40.60% (Azalış)</t>
+          <t>-40.49% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Yahoo + Binance (✓ Doğrulandı)</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1654,46 +1767,46 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1.29</v>
+        <v>1.3</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>-0.52% (Azalış)</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>+0.16% (Artış)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>-1.19% (Azalış)</t>
+          <t>-2.54% (Azalış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-13.41% (Azalış)</t>
+          <t>-14.44% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-12.06% (Azalış)</t>
+          <t>-14.56% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-30.04% (Azalış)</t>
+          <t>-29.31% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-48.67% (Azalış)</t>
+          <t>-49.91% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Yahoo + Binance (✓ Doğrulandı)</t>
+          <t>Yahoo Finance (Birincil)</t>
         </is>
       </c>
     </row>
@@ -1714,7 +1827,7 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>49.69</v>
+        <v>49.72</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -1723,32 +1836,32 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>-0.08% (Yatay)</t>
+          <t>-0.03% (Yatay)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>+0.33% (Artış)</t>
+          <t>+0.39% (Artış)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>+1.51% (Artış)</t>
+          <t>+1.57% (Artış)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>+4.87% (Artış)</t>
+          <t>+4.92% (Artış)</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>+15.68% (Artış)</t>
+          <t>+15.75% (Artış)</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+18.37% (Artış)</t>
+          <t>+18.44% (Artış)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1774,7 +1887,7 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55.67</v>
+        <v>55.75</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -1783,32 +1896,32 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>-0.32% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>+0.16% (Yatay)</t>
+          <t>-0.19% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>+0.30% (Artış)</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>-0.03% (Yatay)</t>
+          <t>+0.11% (Yatay)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>+3.20% (Artış)</t>
+          <t>+3.34% (Artış)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>+10.02% (Artış)</t>
+          <t>+10.17% (Artış)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>+13.98% (Artış)</t>
+          <t>+14.14% (Artış)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1928,7 +2041,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>+2.89% (Artış)</t>
+          <t>+3.07% (Artış)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2314,41 +2427,41 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>116.72</v>
+        <v>111.7</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>+3.14% (Artış)</t>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>-1.30% (Azalış)</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>+6.24% (Artış)</t>
+          <t>+1.67% (Artış)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>+9.49% (Artış)</t>
+          <t>+4.78% (Artış)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>+32.10% (Artış)</t>
+          <t>+26.41% (Artış)</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>+91.82% (Artış)</t>
+          <t>+83.57% (Artış)</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>+77.01% (Artış)</t>
+          <t>+70.22% (Artış)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2365,16 +2478,16 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>CL=F</t>
+          <t>HG=F</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Ham Petrol (WTI)</t>
+          <t>Bakır (Dr. Copper)</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>103.27</v>
+        <v>6.51</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -2383,37 +2496,37 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>+3.82% (Artış)</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+1.83% (Artış)</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>+9.15% (Artış)</t>
+          <t>+2.28% (Artış)</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>-0.36% (Azalış)</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>-3.14% (Azalış)</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>+25.01% (Artış)</t>
+          <t>+2.66% (Artış)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>+79.85% (Artış)</t>
+          <t>+15.59% (Artış)</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>+67.92% (Artış)</t>
+          <t>+26.59% (Artış)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Enerji</t>
+          <t>Sanayi Metali</t>
         </is>
       </c>
     </row>
@@ -2425,55 +2538,55 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>NG=F</t>
+          <t>ZW=F</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Doğalgaz</t>
+          <t>Buğday</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>2.64</v>
+        <v>625</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>-5.58% (Azalış)</t>
+          <t>cent</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>+0.04% (Yatay)</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>-15.28% (Azalış)</t>
+          <t>-5.37% (Azalış)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-19.93% (Azalış)</t>
+          <t>-11.60% (Azalış)</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>-4.59% (Azalış)</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>-28.38% (Azalış)</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>-20.10% (Azalış)</t>
+          <t>-5.30% (Azalış)</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>+23.27% (Artış)</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>+18.82% (Artış)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Enerji</t>
+          <t>Tarım Emtiası</t>
         </is>
       </c>
     </row>
@@ -2485,295 +2598,175 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>HG=F</t>
+          <t>KC=F</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Bakır (Dr. Copper)</t>
+          <t>Kahve</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>6.48</v>
+        <v>306</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>+1.78% (Artış)</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>-0.84% (Azalış)</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>-3.61% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>+2.16% (Artış)</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>+15.03% (Artış)</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>+27.14% (Artış)</t>
+          <t>cent</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>-2.06% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>+0.13% (Yatay)</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>+11.13% (Artış)</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>-5.72% (Azalış)</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>-12.26% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>-21.56% (Azalış)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Sanayi Metali</t>
+          <t>Tarım Emtiası</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Petrol &amp; Emtia</t>
+          <t>Altın &amp; Gümüş (TL / Rasyo)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>ZW=F</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>Buğday</t>
+          <t>GRAM_ALTIN_TL</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Gram Altın (Sadece Günlük TL)</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>625</v>
+        <v>6406.36</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>cent</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>+0.04% (Yatay)</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>-5.37% (Azalış)</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>-11.60% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>-5.30% (Azalış)</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>+23.27% (Artış)</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>+21.95% (Artış)</t>
+          <t>TL</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>-1.32% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Sadece Günlük TL</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Sadece Günlük TL</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Sadece Günlük TL</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Sadece Günlük TL</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Sadece Günlük TL</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>Tarım Emtiası</t>
+          <t>Ons × USD/TRY</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Petrol &amp; Emtia</t>
+          <t>Altın &amp; Gümüş (TL / Rasyo)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>KC=F</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Kahve</t>
+          <t>XAU_XAG</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Altın / Gümüş Oranı (Rasyo)</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>307.45</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>cent</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>-1.60% (Azalış)</t>
+          <t>Kat</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>+0.20% (Artış)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>+0.61% (Artış)</t>
+          <t>+1.27% (Artış)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>+11.66% (Artış)</t>
-        </is>
-      </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>-5.27% (Azalış)</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>-11.84% (Azalış)</t>
+          <t>+9.69% (Artış)</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>+20.02% (Artış)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>-23.71% (Azalış)</t>
+          <t>-13.95% (Azalış)</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Tarım Emtiası</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Altın &amp; Gümüş (TL / Rasyo)</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>GRAM_ALTIN_TL</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>Gram Altın (Sadece Günlük TL)</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>6402.74</v>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>TL</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>-1.38% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>Sadece Günlük TL</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Sadece Günlük TL</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Sadece Günlük TL</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Sadece Günlük TL</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Sadece Günlük TL</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>Ons × USD/TRY</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Altın &amp; Gümüş (TL / Rasyo)</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>XAU_XAG</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Altın / Gümüş Oranı (Rasyo)</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>74.62</v>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>Kat</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>+0.65% (Artış)</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>+1.72% (Artış)</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>+10.17% (Artış)</t>
-        </is>
-      </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>+20.55% (Artış)</t>
-        </is>
-      </c>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>-12.76% (Azalış)</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>Altın/Gümüş oranı 74.62 ile dengeli bantta seyrediyor.</t>
+          <t>Altın/Gümüş oranı 74.29 ile dengeli bantta seyrediyor.</t>
         </is>
       </c>
     </row>
@@ -2837,11 +2830,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>223.73</v>
+        <v>223.54</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TL: 11117.0 / Kur: 49.69</t>
+          <t>TL: 11117.0 / Kur: 49.72</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2863,7 +2856,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>%-0.84</t>
+          <t>%-0.92</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2890,7 +2883,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>%-5.48</t>
+          <t>%-5.56</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2917,7 +2910,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>%-15.03</t>
+          <t>%-15.1</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2944,7 +2937,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>%-22.55</t>
+          <t>%-22.62</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2971,7 +2964,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>%-14.67</t>
+          <t>%-14.74</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2998,7 +2991,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>%-11.36</t>
+          <t>%-11.43</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3033,7 +3026,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Zirveden %-32.9 aşağıda</t>
+          <t>Zirveden %-32.96 aşağıda</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3042,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>223.73</v>
+        <v>223.54</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -3110,7 +3103,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tavana uzaklık: %-26.66</t>
+          <t>Tavana uzaklık: %-26.73</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3119,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>223.73</v>
+        <v>223.54</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -3160,7 +3153,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: %-25.21</t>
+          <t>Uzaklık: %-25.28</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3178,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: +%-8.19</t>
+          <t>Uzaklık: +%-8.26</t>
         </is>
       </c>
     </row>
@@ -3201,7 +3194,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>265.64</v>
+        <v>265.52</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -3226,7 +3219,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>278.58</v>
+        <v>278.49</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -3251,7 +3244,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>291.53</v>
+        <v>291.46</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -3335,7 +3328,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BIST 100 Dolar bazında 223.73$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.0) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.9 aşağıda, 52 haftalık dibinden (223.73$) ise %0.0 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (296.06$) altında baskı altında seyrederken RSI(14) göstergesi 25.5 seviyesindedir.</t>
+          <t>BIST 100 Dolar bazında 223.54$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.0) yer alıyor. 52 haftalık zirvesinden (333.44$) %33.0 aşağıda, 52 haftalık dibinden (223.54$) ise %0.0 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (296.06$) altında baskı altında seyrederken RSI(14) göstergesi 25.5 seviyesindedir.</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -4894,27 +4887,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Orta</t>
+          <t>Yüksek</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Ekonomik Güven Endeksi ve Dış Ticaret Dengesi</t>
+          <t>Fed Faiz Kararı</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -4924,12 +4917,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.00%</t>
         </is>
       </c>
     </row>
@@ -4941,27 +4934,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Orta</t>
+          <t>Yüksek</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Ekonomik Güven Endeksi ve Dış Ticaret Dengesi</t>
+          <t>Fed (FOMC) Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -4988,12 +4981,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -5008,7 +5001,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Durable Goods Orders MoM</t>
+          <t>Fed Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -5018,12 +5011,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>0.6</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5035,12 +5028,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -5055,7 +5048,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Fed Interest Rate Decision</t>
+          <t>Öncü GSYH Büyüme Oranı (Çeyreklik)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -5065,12 +5058,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1.5%</t>
         </is>
       </c>
     </row>
@@ -5082,12 +5075,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -5102,7 +5095,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Fed Press Conference</t>
+          <t>Çekirdek PCE Enflasyon Endeksi (Aylık)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -5112,12 +5105,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.3%</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.2%</t>
         </is>
       </c>
     </row>
@@ -5134,12 +5127,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -5149,7 +5142,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Personal Income MoM</t>
+          <t>Avrupa Merkez Bankası (ECB) Faiz Kararı</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5159,12 +5152,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>2.65%</t>
         </is>
       </c>
     </row>
@@ -5181,12 +5174,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -5196,7 +5189,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Personal Spending MoM</t>
+          <t>ECB Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5206,12 +5199,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>0.9</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5228,12 +5221,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -5243,7 +5236,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Core PCE Price Index MoM</t>
+          <t>ECB Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -5253,34 +5246,34 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Gelecek Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-03</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Türkiye (TÜİK)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -5290,7 +5283,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>GDP Growth Rate QoQ Adv</t>
+          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5300,34 +5293,34 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Gelecek Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>Türkiye (TCMB)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -5337,7 +5330,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>ECB Interest Rate Decision</t>
+          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -5347,576 +5340,12 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2.65</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2.65</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Bu Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-29</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>13:15</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Euro Bölgesi (ECB)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Deposit Facility Rate</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Türkiye (TÜİK)</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Türkiye (TÜİK)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Türkiye (TCMB)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-02</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>ABD (Fed/Makro)</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>ISM İmalat PMI</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>54.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>ABD (Fed/Makro)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Midterm Elections</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>ABD (Fed/Makro)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>JOLTs Job Openings</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>7.079</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Euro Bölgesi (ECB)</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Inflation Rate YoY Flash</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>3.8</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-04</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>ABD (Fed/Makro)</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>ISM Hizmetler PMI</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>54.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-06</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>ABD (Fed/Makro)</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>İşsizlik Oranı</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>4.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-06</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>ABD (Fed/Makro)</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Non Farm Payrolls</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-06</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>ABD (Fed/Makro)</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Michigan Consumer Sentiment Prel</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>48</t>
         </is>
       </c>
     </row>
@@ -6024,7 +5453,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>51/100 (Nötr)</t>
+          <t>54/100 (Nötr)</t>
         </is>
       </c>
     </row>
@@ -6124,17 +5553,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DW.com</t>
+          <t>Bloomberght</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın faiz indirimi işe yarayacak mı?</t>
+          <t>TCMB'de Ocak'tan bu yana ilk faiz indirimi</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz</t>
+          <t>TCMB, Faiz</t>
         </is>
       </c>
     </row>
@@ -6146,17 +5575,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Bloomberght</t>
+          <t>DW.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Fitch'ten Türk leasing ve faktoring şirketleri için varlık uyarısı</t>
+          <t>Merkez Bankası'nın faiz indirimi işe yarayacak mı?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Fitch</t>
+          <t>Merkez Bankası, Faiz</t>
         </is>
       </c>
     </row>
@@ -6168,17 +5597,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Habertürk</t>
+          <t>Bloomberght</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan, Türkiye'deki bankacılık faaliyetlerini büyütme kararı aldığını açıkladı</t>
+          <t>Fitch'ten Türk leasing ve faktoring şirketleri için varlık uyarısı</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan</t>
+          <t>Fitch</t>
         </is>
       </c>
     </row>
@@ -6190,17 +5619,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Uzmanpara</t>
+          <t>Habertürk</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>EKİM 2026 FED FAİZ KARARI NE ZAMAN AÇIKLANACAK? Amerikan Merkez Bankası (FED) faiz beklentisi ne yönde? FED Ekim ayı toplantı tarihleri...</t>
+          <t>JPMorgan, Türkiye'deki bankacılık faaliyetlerini büyütme kararı aldığını açıkladı</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Fed, Faiz</t>
+          <t>JPMorgan</t>
         </is>
       </c>
     </row>
@@ -6212,17 +5641,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CNN Türk</t>
+          <t>Uzmanpara</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>FED FAİZ KARARI NE ZAMAN, BU HAFTA MI? FED Ekim Ayı Faiz Kararı Toplantı Tarihi 2026</t>
+          <t>EKİM 2026 FED FAİZ KARARI NE ZAMAN AÇIKLANACAK? Amerikan Merkez Bankası (FED) faiz beklentisi ne yönde? FED Ekim ayı toplantı tarihleri...</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Fed, Faiz</t>
+          <t>Merkez Bankası, Fed, Faiz</t>
         </is>
       </c>
     </row>
@@ -6239,7 +5668,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Fed'in faiz kararı öncesi altın fiyatları üzerinde baskı sürüyor</t>
+          <t>Haftaya Bakış: Gözler Fed'in faiz kararında, dev şirketlerin bilançolarında olacak</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -6278,12 +5707,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Gazete Merhaba</t>
+          <t>Olay Gazetesi Bursa</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Balıkesir'de Eylül'de 3 Bin Konut Satıldı</t>
+          <t>Konut satış rakamları açıklandı - Olay Gazetesi Bursa</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
📊 Otomatik Günlük Finans Raporu ve Excel Güncellemesi (2026-10-26)
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI3"/>
+  <dimension ref="A1:AI4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -940,6 +940,119 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>11151.96</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>224.35</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>-32.72</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>295.79</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>7676.77</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>4026.8</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>6435.55</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>53.98</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>86.27</v>
+      </c>
+      <c r="O4" s="2" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="P4" s="2" t="n">
+        <v>49.71</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>55.64</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="S4" s="2" t="n">
+        <v>102.03</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="U4" s="2" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="V4" s="2" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="W4" s="2" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="X4" s="2" t="n">
+        <v>79697.81</v>
+      </c>
+      <c r="Y4" s="2" t="n">
+        <v>2305.2</v>
+      </c>
+      <c r="Z4" s="2" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="AA4" s="2" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="AB4" s="2" t="n">
+        <v>59.43</v>
+      </c>
+      <c r="AC4" s="2" t="n">
+        <v>110.18</v>
+      </c>
+      <c r="AD4" s="2" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="AE4" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="AF4" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="AG4" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>TI2 (%2.42)</t>
+        </is>
+      </c>
+      <c r="AI4" s="2" t="inlineStr">
+        <is>
+          <t>IIH (%74.5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1047,41 +1160,41 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>11117</v>
+        <v>11151.96</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>-0.92% (Azalış)</t>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>+0.31% (Artış)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>-5.16% (Azalış)</t>
+          <t>-2.43% (Azalış)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>-13.74% (Azalış)</t>
+          <t>-13.55% (Azalış)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>-18.78% (Azalış)</t>
+          <t>-17.40% (Azalış)</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>-1.28% (Azalış)</t>
+          <t>-0.97% (Azalış)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>+4.80% (Artış)</t>
+          <t>+2.75% (Artış)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -1107,41 +1220,41 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13874.2</v>
+        <v>13948.59</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>-0.98% (Azalış)</t>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>+0.54% (Artış)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>-4.70% (Azalış)</t>
+          <t>-1.92% (Azalış)</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>-12.96% (Azalış)</t>
+          <t>-12.53% (Azalış)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>-10.47% (Azalış)</t>
+          <t>-8.90% (Azalış)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>+13.50% (Artış)</t>
+          <t>+14.11% (Artış)</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>+19.94% (Artış)</t>
+          <t>+17.60% (Artış)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -1167,41 +1280,41 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>15107.2</v>
+        <v>15406.16</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>-1.58% (Azalış)</t>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>+1.98% (Artış)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>-4.47% (Azalış)</t>
+          <t>-2.85% (Azalış)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>-7.12% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>-2.14% (Azalış)</t>
+          <t>-5.30% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>+3.06% (Artış)</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>-8.66% (Azalış)</t>
+          <t>-6.86% (Azalış)</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>+7.21% (Artış)</t>
+          <t>+6.72% (Artış)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1227,41 +1340,41 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13562</v>
+        <v>13582.95</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>-1.69% (Azalış)</t>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>+0.15% (Artış)</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>-8.47% (Azalış)</t>
+          <t>-4.98% (Azalış)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>-21.67% (Azalış)</t>
+          <t>-21.57% (Azalış)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>-27.76% (Azalış)</t>
+          <t>-26.53% (Azalış)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>-3.22% (Azalış)</t>
+          <t>-3.07% (Azalış)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>-1.34% (Azalış)</t>
+          <t>-3.63% (Azalış)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1287,41 +1400,41 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7623.68</v>
+        <v>7676.77</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>-0.52% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>-0.47% (Azalış)</t>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>+0.70% (Artış)</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>-0.18% (Yatay)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>-1.04% (Azalış)</t>
+          <t>-0.86% (Azalış)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>+2.84% (Artış)</t>
+          <t>+3.34% (Artış)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>+11.37% (Artış)</t>
+          <t>+12.14% (Artış)</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>+12.25% (Artış)</t>
+          <t>+11.66% (Artış)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1347,41 +1460,41 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>25955.34</v>
+        <v>26169.38</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>-0.21% (Azalış)</t>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>+0.82% (Artış)</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>-0.71% (Azalış)</t>
+          <t>-0.99% (Azalış)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>-3.65% (Azalış)</t>
+          <t>-3.32% (Azalış)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>+4.10% (Artış)</t>
+          <t>+5.20% (Artış)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>+11.67% (Artış)</t>
+          <t>+12.60% (Artış)</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>+11.85% (Artış)</t>
+          <t>+10.71% (Artış)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1407,41 +1520,41 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>52215.16</v>
+        <v>52361.58</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>-1.23% (Azalış)</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>+0.28% (Artış)</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>+0.41% (Artış)</t>
+          <t>+0.76% (Artış)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>+1.68% (Artış)</t>
+          <t>+1.03% (Artış)</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>+0.01% (Yatay)</t>
+          <t>-0.73% (Yatay)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>+8.64% (Artış)</t>
+          <t>+8.94% (Artış)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>+10.61% (Artış)</t>
+          <t>+10.13% (Artış)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1467,41 +1580,41 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>19.45</v>
+        <v>18.39</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>+2.21% (Artış)</t>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>-5.45% (Azalış)</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>-2.70% (Azalış)</t>
+          <t>-0.27% (Azalış)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>+24.12% (Artış)</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>+6.81% (Artış)</t>
+          <t>+23.67% (Artış)</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>-10.99% (Azalış)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>+30.10% (Artış)</t>
+          <t>+23.01% (Artış)</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>+12.43% (Artış)</t>
+          <t>+16.47% (Artış)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1527,41 +1640,41 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>4007.9</v>
+        <v>4026.8</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>-1.29% (Azalış)</t>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>+0.47% (Artış)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>-4.14% (Azalış)</t>
+          <t>-3.20% (Azalış)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>-6.75% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>-1.69% (Azalış)</t>
+          <t>-6.81% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>-0.29% (Yatay)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>-7.68% (Azalış)</t>
+          <t>-7.24% (Azalış)</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>-0.29% (Yatay)</t>
+          <t>+0.18% (Yatay)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1587,41 +1700,41 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>53.95</v>
+        <v>53.98</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>-1.49% (Azalış)</t>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>+0.50% (Artış)</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>-5.34% (Azalış)</t>
+          <t>-5.26% (Azalış)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-14.98% (Azalış)</t>
+          <t>-15.98% (Azalış)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>-7.74% (Azalış)</t>
+          <t>-5.79% (Azalış)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>-23.08% (Azalış)</t>
+          <t>-23.03% (Azalış)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+15.86% (Artış)</t>
+          <t>+15.93% (Artış)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1647,7 +1760,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>80564.78</v>
+        <v>79697.81</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1656,32 +1769,32 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>-0.28% (Azalış)</t>
+          <t>-0.41% (Azalış)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>-2.86% (Azalış)</t>
+          <t>-5.14% (Azalış)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-6.84% (Azalış)</t>
+          <t>-7.10% (Azalış)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>+3.61% (Artış)</t>
+          <t>+0.93% (Artış)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-7.94% (Azalış)</t>
+          <t>-8.93% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-27.84% (Azalış)</t>
+          <t>-30.38% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1707,7 +1820,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2352.71</v>
+        <v>2305.2</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -1716,32 +1829,32 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>-0.14% (Azalış)</t>
+          <t>-0.93% (Azalış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-3.84% (Azalış)</t>
+          <t>-6.70% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-13.71% (Azalış)</t>
+          <t>-14.97% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-4.51% (Azalış)</t>
+          <t>-7.12% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-20.71% (Azalış)</t>
+          <t>-22.31% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-40.49% (Azalış)</t>
+          <t>-44.56% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1767,41 +1880,41 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1.3</v>
+        <v>1.29</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>+0.16% (Artış)</t>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>-0.43% (Azalış)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>-2.54% (Azalış)</t>
+          <t>-5.48% (Azalış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-14.44% (Azalış)</t>
+          <t>-14.50% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-14.56% (Azalış)</t>
+          <t>-12.86% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-29.31% (Azalış)</t>
+          <t>-29.95% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-49.91% (Azalış)</t>
+          <t>-51.27% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1827,7 +1940,7 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>49.72</v>
+        <v>49.71</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -1836,32 +1949,32 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>-0.03% (Yatay)</t>
+          <t>-0.04% (Yatay)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>+0.39% (Artış)</t>
+          <t>+0.38% (Artış)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>+1.57% (Artış)</t>
+          <t>+1.55% (Artış)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>+4.92% (Artış)</t>
+          <t>+4.91% (Artış)</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>+15.75% (Artış)</t>
+          <t>+15.73% (Artış)</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+18.44% (Artış)</t>
+          <t>+18.38% (Artış)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1887,7 +2000,7 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55.75</v>
+        <v>55.64</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -1896,32 +2009,32 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>-0.19% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>+0.30% (Artış)</t>
+          <t>-0.38% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>+0.11% (Yatay)</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>+0.11% (Yatay)</t>
+          <t>-0.08% (Yatay)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>+3.34% (Artış)</t>
+          <t>+3.14% (Artış)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>+10.17% (Artış)</t>
+          <t>+9.96% (Artış)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>+14.14% (Artış)</t>
+          <t>+13.81% (Artış)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -1956,32 +2069,32 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>-0.15% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-0.19% (Yatay)</t>
+          <t>-0.40% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>-0.43% (Azalış)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-1.50% (Azalış)</t>
+          <t>-1.74% (Azalış)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>-1.60% (Azalış)</t>
+          <t>-1.84% (Azalış)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>-4.62% (Azalış)</t>
+          <t>-4.86% (Azalış)</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>-3.48% (Azalış)</t>
+          <t>-3.91% (Azalış)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2007,7 +2120,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>101.81</v>
+        <v>102.03</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -2016,32 +2129,32 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>+0.20% (Artış)</t>
+          <t>+0.21% (Artış)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>-0.03% (Yatay)</t>
+          <t>+0.05% (Yatay)</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>+0.51% (Artış)</t>
+          <t>+1.05% (Artış)</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>+0.30% (Yatay)</t>
+          <t>+0.64% (Yatay)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>+3.59% (Artış)</t>
+          <t>+3.81% (Artış)</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>+3.07% (Artış)</t>
+          <t>+3.29% (Artış)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2067,7 +2180,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>4.8</v>
+        <v>4.82</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -2076,32 +2189,32 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>+0.78% (Artış)</t>
+          <t>+0.40% (Artış)</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>-1.92% (Azalış)</t>
+          <t>-2.13% (Azalış)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>-4.38% (Azalış)</t>
+          <t>-3.65% (Azalış)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>+9.28% (Artış)</t>
+          <t>+10.62% (Artış)</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>+29.10% (Artış)</t>
+          <t>+29.61% (Artış)</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>+33.58% (Artış)</t>
+          <t>+33.48% (Artış)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -2134,34 +2247,34 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>+0.71% (Artış)</t>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>-0.04% (Yatay)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>-2.16% (Azalış)</t>
+          <t>-2.92% (Azalış)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>-3.37% (Azalış)</t>
+          <t>-3.82% (Azalış)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>+7.48% (Artış)</t>
+          <t>+8.30% (Artış)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>+19.82% (Artış)</t>
+          <t>+19.77% (Artış)</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>+24.98% (Artış)</t>
+          <t>+24.74% (Artış)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2187,41 +2300,41 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>5.32</v>
+        <v>5.3</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>+0.53% (Artış)</t>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>-0.26% (Azalış)</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>-2.23% (Azalış)</t>
+          <t>-3.13% (Azalış)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>-2.67% (Azalış)</t>
+          <t>-3.69% (Azalış)</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>+3.71% (Artış)</t>
+          <t>+4.02% (Artış)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>+9.81% (Artış)</t>
+          <t>+9.52% (Artış)</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>+16.23% (Artış)</t>
+          <t>+16.00% (Artış)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2427,7 +2540,7 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>111.7</v>
+        <v>110.18</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -2436,32 +2549,32 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>-1.30% (Azalış)</t>
+          <t>-5.60% (Azalış)</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>+1.67% (Artış)</t>
+          <t>+0.58% (Artış)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>+4.78% (Artış)</t>
+          <t>+5.62% (Artış)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>+26.41% (Artış)</t>
+          <t>+31.03% (Artış)</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>+83.57% (Artış)</t>
+          <t>+81.07% (Artış)</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>+70.22% (Artış)</t>
+          <t>+67.91% (Artış)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2487,7 +2600,7 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>6.51</v>
+        <v>6.55</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -2496,32 +2609,32 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>+2.28% (Artış)</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>-0.36% (Azalış)</t>
+          <t>+1.10% (Artış)</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>+0.14% (Yatay)</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>-3.14% (Azalış)</t>
+          <t>-2.22% (Azalış)</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>+2.66% (Artış)</t>
+          <t>+3.56% (Artış)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>+15.59% (Artış)</t>
+          <t>+16.29% (Artış)</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>+26.59% (Artış)</t>
+          <t>+27.36% (Artış)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2547,41 +2660,41 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>625</v>
+        <v>615.5</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>cent</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>+0.04% (Yatay)</t>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>-1.52% (Azalış)</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>-5.37% (Azalış)</t>
+          <t>-6.07% (Azalış)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-11.60% (Azalış)</t>
+          <t>-12.48% (Azalış)</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>-5.30% (Azalış)</t>
+          <t>-7.09% (Azalış)</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>+23.27% (Artış)</t>
+          <t>+21.40% (Artış)</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>+18.82% (Artış)</t>
+          <t>+17.02% (Artış)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2607,7 +2720,7 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>306</v>
+        <v>299.5</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -2616,32 +2729,32 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>-2.06% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>+0.13% (Yatay)</t>
+          <t>-2.59% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>-5.13% (Azalış)</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>+11.13% (Artış)</t>
+          <t>+7.50% (Artış)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>-5.72% (Azalış)</t>
+          <t>-11.76% (Azalış)</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>-12.26% (Azalış)</t>
+          <t>-14.12% (Azalış)</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>-21.56% (Azalış)</t>
+          <t>-23.22% (Azalış)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2667,16 +2780,16 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>6406.36</v>
+        <v>6435.55</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>-1.32% (Azalış)</t>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>+0.43% (Artış)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2727,26 +2840,26 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>74.29000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Kat</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>+0.20% (Artış)</t>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>-0.03% (Yatay)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>+1.27% (Artış)</t>
+          <t>+2.16% (Artış)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>+9.69% (Artış)</t>
+          <t>+10.91% (Artış)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2756,17 +2869,17 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>+20.02% (Artış)</t>
+          <t>+20.52% (Artış)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>-13.95% (Azalış)</t>
+          <t>-13.59% (Azalış)</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Altın/Gümüş oranı 74.29 ile dengeli bantta seyrediyor.</t>
+          <t>Altın/Gümüş oranı 74.60 ile dengeli bantta seyrediyor.</t>
         </is>
       </c>
     </row>
@@ -2830,11 +2943,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>223.54</v>
+        <v>224.35</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TL: 11117.0 / Kur: 49.72</t>
+          <t>TL: 11151.96 / Kur: 49.71</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2856,7 +2969,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>%-0.92</t>
+          <t>%0.36</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2866,7 +2979,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Azalış</t>
+          <t>Artış</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2996,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>%-5.56</t>
+          <t>%-2.71</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2910,7 +3023,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>%-15.1</t>
+          <t>%-14.87</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2937,7 +3050,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>%-22.62</t>
+          <t>%-21.29</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -2964,7 +3077,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>%-14.74</t>
+          <t>%-14.43</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -2991,7 +3104,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>%-11.43</t>
+          <t>%-13.2</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3026,7 +3139,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Zirveden %-32.96 aşağıda</t>
+          <t>Zirveden %-32.72 aşağıda</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3164,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dipten +%0.0 yukarıda</t>
+          <t>Dipten +%0.36 yukarıda</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3181,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>%0.0</t>
+          <t>%0.7</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3103,7 +3216,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tavana uzaklık: %-26.73</t>
+          <t>Tavana uzaklık: %-26.46</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3241,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Tabandan uzaklık: +%0.0</t>
+          <t>Tabandan uzaklık: +%0.36</t>
         </is>
       </c>
     </row>
@@ -3153,7 +3266,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: %-25.28</t>
+          <t>Uzaklık: %-25.01</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3291,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: +%-8.26</t>
+          <t>Uzaklık: +%-7.93</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3382,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>271.17</v>
+        <v>269.75</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -3294,7 +3407,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>296.06</v>
+        <v>295.79</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -3319,7 +3432,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>25.5</v>
+        <v>26.6</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -3328,7 +3441,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BIST 100 Dolar bazında 223.54$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.0) yer alıyor. 52 haftalık zirvesinden (333.44$) %33.0 aşağıda, 52 haftalık dibinden (223.54$) ise %0.0 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (296.06$) altında baskı altında seyrederken RSI(14) göstergesi 25.5 seviyesindedir.</t>
+          <t>BIST 100 Dolar bazında 224.35$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.7) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.7 aşağıda, 52 haftalık dibinden (223.54$) ise %0.4 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.79$) altında baskı altında seyrederken RSI(14) göstergesi 26.6 seviyesindedir.</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5479,7 @@
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="75" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -5409,7 +5522,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>21/100 (Aşırı Korku)</t>
+          <t>27/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5431,7 +5544,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>26/100 (Korku)</t>
+          <t>28/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5453,7 +5566,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>54/100 (Nötr)</t>
+          <t>50/100 (Nötr)</t>
         </is>
       </c>
     </row>
@@ -5553,12 +5666,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Bloomberght</t>
+          <t>Euronews.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TCMB'de Ocak'tan bu yana ilk faiz indirimi</t>
+          <t>TCMB faiz kararını açıkladı: Ocaktan bu yana ilk faiz indirimi</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -5575,17 +5688,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DW.com</t>
+          <t>Anadolu Ajansı</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın faiz indirimi işe yarayacak mı?</t>
+          <t>Üç büyük merkez bankası enflasyon riskleri altında faiz kararı alacak</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz</t>
+          <t>Merkez Bankası, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -5597,17 +5710,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Bloomberght</t>
+          <t>Habertürk</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Fitch'ten Türk leasing ve faktoring şirketleri için varlık uyarısı</t>
+          <t>JPMorgan, Türkiye'deki bankacılık faaliyetlerini büyütme kararı aldığını açıkladı</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Fitch</t>
+          <t>JPMorgan</t>
         </is>
       </c>
     </row>
@@ -5619,17 +5732,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Habertürk</t>
+          <t>Uzmanpara</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan, Türkiye'deki bankacılık faaliyetlerini büyütme kararı aldığını açıkladı</t>
+          <t>GÖZLER FED'İN FAİZ KARARINA ÇEVRİLDİ! FED toplantısı ne zaman, faiz kararı hangi gün saat kaçta açıklanacak? Amerikan Merkez Bankası (FED) Ekim ayı faiz beklentisi ne yönde?</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan</t>
+          <t>Merkez Bankası, Fed, Faiz</t>
         </is>
       </c>
     </row>
@@ -5641,17 +5754,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Uzmanpara</t>
+          <t>CNBC-e</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>EKİM 2026 FED FAİZ KARARI NE ZAMAN AÇIKLANACAK? Amerikan Merkez Bankası (FED) faiz beklentisi ne yönde? FED Ekim ayı toplantı tarihleri...</t>
+          <t>ECB faiz kararı öncesi 5 kritik soru: Piyasalar ne bekliyor?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Fed, Faiz</t>
+          <t>ECB, Faiz</t>
         </is>
       </c>
     </row>
@@ -5663,12 +5776,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Foreks.com</t>
+          <t>Platin Dergisi</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Haftaya Bakış: Gözler Fed'in faiz kararında, dev şirketlerin bilançolarında olacak</t>
+          <t>Fed faiz kararı ne zaman? Beklentiler ne yönde?</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -5707,12 +5820,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Olay Gazetesi Bursa</t>
+          <t>Son Dakika</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Konut satış rakamları açıklandı - Olay Gazetesi Bursa</t>
+          <t>TÜİK'e göre Uşak'ta Eylül'de satılan konut sayısı 52 artışla 770'e ulaştı</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
📊 Otomatik Günlük Finans Raporu ve Excel Güncellemesi (2026-10-27)
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI4"/>
+  <dimension ref="A1:AI5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1053,6 +1053,119 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>11151.03</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>223.99</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>-32.82</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>295.5</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>7722.6</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>4072.7</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>6518.54</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>54.46</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>87.17</v>
+      </c>
+      <c r="O5" s="2" t="n">
+        <v>74.78</v>
+      </c>
+      <c r="P5" s="2" t="n">
+        <v>49.78</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>55.48</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="S5" s="2" t="n">
+        <v>102.33</v>
+      </c>
+      <c r="T5" s="2" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="U5" s="2" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="V5" s="2" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="W5" s="2" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="X5" s="2" t="n">
+        <v>80666.64999999999</v>
+      </c>
+      <c r="Y5" s="2" t="n">
+        <v>2343.52</v>
+      </c>
+      <c r="Z5" s="2" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="AA5" s="2" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="AB5" s="2" t="n">
+        <v>59.45</v>
+      </c>
+      <c r="AC5" s="2" t="n">
+        <v>109.84</v>
+      </c>
+      <c r="AD5" s="2" t="n">
+        <v>6.66</v>
+      </c>
+      <c r="AE5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="AF5" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="AG5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>TI2 (%2.42)</t>
+        </is>
+      </c>
+      <c r="AI5" s="2" t="inlineStr">
+        <is>
+          <t>IIH (%74.5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1160,41 +1273,41 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>11151.96</v>
+        <v>11151.03</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>+0.31% (Artış)</t>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>-0.01% (Yatay)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>-2.43% (Azalış)</t>
+          <t>-5.48% (Azalış)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>-13.55% (Azalış)</t>
+          <t>-11.45% (Azalış)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>-17.40% (Azalış)</t>
+          <t>-16.11% (Azalış)</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>-0.97% (Azalış)</t>
+          <t>-0.98% (Azalış)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>+2.75% (Artış)</t>
+          <t>+2.74% (Artış)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -1220,41 +1333,41 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13948.59</v>
+        <v>13934.73</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>+0.54% (Artış)</t>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>-0.10% (Yatay)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>-1.92% (Azalış)</t>
+          <t>-5.05% (Azalış)</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>-12.53% (Azalış)</t>
+          <t>-10.95% (Azalış)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>-8.90% (Azalış)</t>
+          <t>-7.31% (Azalış)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>+14.11% (Artış)</t>
+          <t>+14.00% (Artış)</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>+17.60% (Artış)</t>
+          <t>+17.48% (Artış)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -1280,41 +1393,41 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>15406.16</v>
+        <v>15313.58</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>+1.98% (Artış)</t>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>-0.60% (Azalış)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>-2.85% (Azalış)</t>
+          <t>-5.17% (Azalış)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>-5.30% (Azalış)</t>
+          <t>-5.02% (Azalış)</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>+3.06% (Artış)</t>
+          <t>+4.97% (Artış)</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>-6.86% (Azalış)</t>
+          <t>-7.41% (Azalış)</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>+6.72% (Artış)</t>
+          <t>+6.08% (Artış)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1340,7 +1453,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13582.95</v>
+        <v>13656.29</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -1349,32 +1462,32 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>+0.15% (Artış)</t>
+          <t>+0.54% (Artış)</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>-4.98% (Azalış)</t>
+          <t>-6.73% (Azalış)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>-21.57% (Azalış)</t>
+          <t>-17.76% (Azalış)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>-26.53% (Azalış)</t>
+          <t>-25.65% (Azalış)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>-3.07% (Azalış)</t>
+          <t>-2.55% (Azalış)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>-3.63% (Azalış)</t>
+          <t>-3.11% (Azalış)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1400,7 +1513,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7676.77</v>
+        <v>7722.6</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -1409,32 +1522,32 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>+0.70% (Artış)</t>
+          <t>+0.60% (Artış)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>-0.18% (Yatay)</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>-0.86% (Azalış)</t>
+          <t>+0.13% (Yatay)</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>+0.51% (Artış)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>+3.34% (Artış)</t>
+          <t>+5.56% (Artış)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>+12.14% (Artış)</t>
+          <t>+12.81% (Artış)</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>+11.66% (Artış)</t>
+          <t>+12.07% (Artış)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1460,7 +1573,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>26169.38</v>
+        <v>26477.81</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -1469,32 +1582,32 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>+0.82% (Artış)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>-0.99% (Azalış)</t>
+          <t>+1.18% (Artış)</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>+0.20% (Yatay)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>-3.32% (Azalış)</t>
+          <t>-1.28% (Azalış)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>+5.20% (Artış)</t>
+          <t>+8.32% (Artış)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>+12.60% (Artış)</t>
+          <t>+13.92% (Artış)</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>+10.71% (Artış)</t>
+          <t>+11.12% (Artış)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1520,41 +1633,41 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>52361.58</v>
+        <v>52377.57</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>+0.28% (Artış)</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>+0.76% (Artış)</t>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>+0.03% (Yatay)</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>-0.23% (Yatay)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>+1.03% (Artış)</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>-0.73% (Yatay)</t>
+          <t>+1.74% (Artış)</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>+1.52% (Artış)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>+8.94% (Artış)</t>
+          <t>+8.98% (Artış)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>+10.13% (Artış)</t>
+          <t>+9.79% (Artış)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1580,7 +1693,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>18.39</v>
+        <v>17.57</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -1589,32 +1702,32 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>-5.45% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>-0.27% (Azalış)</t>
+          <t>-4.46% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>+1.50% (Artış)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>+23.67% (Artış)</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>-10.99% (Azalış)</t>
+          <t>+9.33% (Artış)</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>+2.81% (Artış)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>+23.01% (Artış)</t>
+          <t>+17.53% (Artış)</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>+16.47% (Artış)</t>
+          <t>+11.27% (Artış)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1640,7 +1753,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>4026.8</v>
+        <v>4072.7</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -1649,32 +1762,32 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>+0.47% (Artış)</t>
+          <t>+0.85% (Artış)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>-3.20% (Azalış)</t>
+          <t>-1.69% (Azalış)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>-6.81% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>-0.29% (Yatay)</t>
+          <t>-2.30% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>+0.90% (Artış)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>-7.24% (Azalış)</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>+0.18% (Yatay)</t>
+          <t>-6.18% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>+1.32% (Artış)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1700,7 +1813,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>53.98</v>
+        <v>54.46</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -1709,32 +1822,32 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>+0.50% (Artış)</t>
+          <t>+0.65% (Artış)</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>-5.26% (Azalış)</t>
+          <t>-5.63% (Azalış)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-15.98% (Azalış)</t>
+          <t>-11.04% (Azalış)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>-5.79% (Azalış)</t>
+          <t>-5.88% (Azalış)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>-23.03% (Azalış)</t>
+          <t>-22.35% (Azalış)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+15.93% (Artış)</t>
+          <t>+16.96% (Artış)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1760,41 +1873,41 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>79697.81</v>
+        <v>80666.64999999999</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>-0.41% (Azalış)</t>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>+0.82% (Artış)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>-5.14% (Azalış)</t>
+          <t>-0.79% (Azalış)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-7.10% (Azalış)</t>
+          <t>-5.72% (Azalış)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>+0.93% (Artış)</t>
+          <t>+2.68% (Artış)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-8.93% (Azalış)</t>
+          <t>-7.82% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-30.38% (Azalış)</t>
+          <t>-29.31% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1820,41 +1933,41 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2305.2</v>
+        <v>2343.52</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>-0.93% (Azalış)</t>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>+1.00% (Artış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-6.70% (Azalış)</t>
+          <t>-1.79% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-14.97% (Azalış)</t>
+          <t>-13.12% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-7.12% (Azalış)</t>
+          <t>-4.08% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-22.31% (Azalış)</t>
+          <t>-21.01% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-44.56% (Azalış)</t>
+          <t>-43.12% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1880,41 +1993,41 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1.29</v>
+        <v>1.32</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>-0.43% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>-5.48% (Azalış)</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>+1.19% (Artış)</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>+1.14% (Artış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-14.50% (Azalış)</t>
+          <t>-11.68% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-12.86% (Azalış)</t>
+          <t>-7.73% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-29.95% (Azalış)</t>
+          <t>-28.12% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-51.27% (Azalış)</t>
+          <t>-49.80% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1940,7 +2053,7 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>49.71</v>
+        <v>49.78</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
@@ -1949,32 +2062,32 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>-0.04% (Yatay)</t>
+          <t>+0.09% (Yatay)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>+0.38% (Artış)</t>
+          <t>+0.43% (Artış)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>+1.55% (Artış)</t>
+          <t>+1.66% (Artış)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>+4.91% (Artış)</t>
+          <t>+5.09% (Artış)</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>+15.73% (Artış)</t>
+          <t>+15.90% (Artış)</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+18.38% (Artış)</t>
+          <t>+18.55% (Artış)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -2000,7 +2113,7 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55.64</v>
+        <v>55.48</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -2009,32 +2122,32 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>-0.38% (Azalış)</t>
+          <t>-0.63% (Azalış)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>+0.11% (Yatay)</t>
+          <t>-0.23% (Yatay)</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>-0.08% (Yatay)</t>
+          <t>-0.46% (Yatay)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>+3.14% (Artış)</t>
+          <t>+1.99% (Artış)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>+9.96% (Artış)</t>
+          <t>+9.64% (Artış)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>+13.81% (Artış)</t>
+          <t>+13.49% (Artış)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -2060,7 +2173,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1.12</v>
+        <v>1.11</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -2069,32 +2182,32 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>-0.40% (Azalış)</t>
+          <t>-0.73% (Azalış)</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>-0.43% (Azalış)</t>
+          <t>-0.71% (Azalış)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-1.74% (Azalış)</t>
+          <t>-2.13% (Azalış)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>-1.84% (Azalış)</t>
+          <t>-2.89% (Azalış)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>-4.86% (Azalış)</t>
+          <t>-5.20% (Azalış)</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>-3.91% (Azalış)</t>
+          <t>-4.26% (Azalış)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2120,7 +2233,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>102.03</v>
+        <v>102.33</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -2129,32 +2242,32 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>+0.21% (Artış)</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>+0.05% (Yatay)</t>
+          <t>+0.36% (Artış)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>+0.58% (Artış)</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>+1.05% (Artış)</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>+0.64% (Yatay)</t>
+          <t>+1.11% (Artış)</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>+1.51% (Artış)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>+3.81% (Artış)</t>
+          <t>+4.12% (Artış)</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>+3.29% (Artış)</t>
+          <t>+3.59% (Artış)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2180,7 +2293,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>4.82</v>
+        <v>4.84</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -2189,32 +2302,32 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>+0.40% (Artış)</t>
+          <t>+0.33% (Artış)</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>-2.13% (Azalış)</t>
+          <t>-1.93% (Azalış)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>-3.65% (Azalış)</t>
+          <t>-4.50% (Azalış)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>+10.62% (Artış)</t>
+          <t>+11.21% (Artış)</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>+29.61% (Artış)</t>
+          <t>+30.04% (Artış)</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>+33.48% (Artış)</t>
+          <t>+33.92% (Artış)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -2247,34 +2360,34 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>-0.04% (Yatay)</t>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>+0.14% (Artış)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>-2.92% (Azalış)</t>
+          <t>-2.42% (Azalış)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>-3.82% (Azalış)</t>
+          <t>-4.71% (Azalış)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>+8.30% (Artış)</t>
+          <t>+8.03% (Artış)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>+19.77% (Artış)</t>
+          <t>+19.94% (Artış)</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>+24.74% (Artış)</t>
+          <t>+24.92% (Artış)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2307,34 +2420,34 @@
           <t>%</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>-0.26% (Azalış)</t>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>+0.08% (Yatay)</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>-3.13% (Azalış)</t>
+          <t>-2.21% (Azalış)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>-3.69% (Azalış)</t>
+          <t>-4.60% (Azalış)</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>+4.02% (Artış)</t>
+          <t>+3.15% (Artış)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>+9.52% (Artış)</t>
+          <t>+9.61% (Artış)</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>+16.00% (Artış)</t>
+          <t>+16.08% (Artış)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2540,7 +2653,7 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>110.18</v>
+        <v>109.84</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -2549,32 +2662,32 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>-5.60% (Azalış)</t>
+          <t>-5.15% (Azalış)</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>+0.58% (Artış)</t>
+          <t>+0.97% (Artış)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>+5.62% (Artış)</t>
+          <t>+4.33% (Artış)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>+31.03% (Artış)</t>
+          <t>+21.05% (Artış)</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>+81.07% (Artış)</t>
+          <t>+80.51% (Artış)</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>+67.91% (Artış)</t>
+          <t>+67.39% (Artış)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2600,7 +2713,7 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>6.55</v>
+        <v>6.66</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -2609,32 +2722,32 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>+1.10% (Artış)</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>+0.14% (Yatay)</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>-2.22% (Azalış)</t>
+          <t>+2.28% (Artış)</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>+1.37% (Artış)</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>+1.38% (Artış)</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>+3.56% (Artış)</t>
+          <t>+6.11% (Artış)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>+16.29% (Artış)</t>
+          <t>+18.23% (Artış)</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>+27.36% (Artış)</t>
+          <t>+29.49% (Artış)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2660,7 +2773,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>615.5</v>
+        <v>611</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -2669,32 +2782,32 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>-1.52% (Azalış)</t>
+          <t>-0.81% (Azalış)</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>-6.07% (Azalış)</t>
+          <t>-5.01% (Azalış)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-12.48% (Azalış)</t>
+          <t>-11.29% (Azalış)</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>-7.09% (Azalış)</t>
+          <t>-7.53% (Azalış)</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>+21.40% (Artış)</t>
+          <t>+20.51% (Artış)</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>+17.02% (Artış)</t>
+          <t>+16.16% (Artış)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2720,7 +2833,7 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>299.5</v>
+        <v>294.25</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -2729,32 +2842,32 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>-2.59% (Azalış)</t>
+          <t>-2.23% (Azalış)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>-5.13% (Azalış)</t>
+          <t>-5.48% (Azalış)</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>+7.50% (Artış)</t>
+          <t>+1.90% (Artış)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>-11.76% (Azalış)</t>
+          <t>-9.68% (Azalış)</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>-14.12% (Azalış)</t>
+          <t>-15.63% (Azalış)</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>-23.22% (Azalış)</t>
+          <t>-24.57% (Azalış)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2780,7 +2893,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>6435.55</v>
+        <v>6518.54</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -2789,7 +2902,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>+0.43% (Artış)</t>
+          <t>+0.94% (Artış)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2840,26 +2953,26 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>74.59999999999999</v>
+        <v>74.78</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Kat</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>-0.03% (Yatay)</t>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>+0.19% (Artış)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>+2.16% (Artış)</t>
+          <t>+4.16% (Artış)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>+10.91% (Artış)</t>
+          <t>+9.83% (Artış)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2869,17 +2982,17 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>+20.52% (Artış)</t>
+          <t>+20.81% (Artış)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>-13.59% (Azalış)</t>
+          <t>-13.38% (Azalış)</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Altın/Gümüş oranı 74.60 ile dengeli bantta seyrediyor.</t>
+          <t>Altın/Gümüş oranı 74.78 ile dengeli bantta seyrediyor.</t>
         </is>
       </c>
     </row>
@@ -2943,11 +3056,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>224.35</v>
+        <v>223.99</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TL: 11151.96 / Kur: 49.71</t>
+          <t>TL: 11151.03 / Kur: 49.78</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2969,7 +3082,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>%0.36</t>
+          <t>%-0.1</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2979,7 +3092,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Artış</t>
+          <t>Yatay</t>
         </is>
       </c>
     </row>
@@ -2996,7 +3109,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>%-2.71</t>
+          <t>%-5.86</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3023,7 +3136,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>%-14.87</t>
+          <t>%-12.85</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3050,7 +3163,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>%-21.29</t>
+          <t>%-19.96</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -3077,7 +3190,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>%-14.43</t>
+          <t>%-14.57</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -3104,7 +3217,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>%-13.2</t>
+          <t>%-13.34</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3139,7 +3252,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Zirveden %-32.72 aşağıda</t>
+          <t>Zirveden %-32.82 aşağıda</t>
         </is>
       </c>
     </row>
@@ -3164,7 +3277,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dipten +%0.36 yukarıda</t>
+          <t>Dipten +%0.2 yukarıda</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3294,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>%0.7</t>
+          <t>%0.4</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3216,7 +3329,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tavana uzaklık: %-26.46</t>
+          <t>Tavana uzaklık: %-26.58</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3354,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Tabandan uzaklık: +%0.36</t>
+          <t>Tabandan uzaklık: +%0.2</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3379,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: %-25.01</t>
+          <t>Uzaklık: %-25.13</t>
         </is>
       </c>
     </row>
@@ -3291,7 +3404,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: +%-7.93</t>
+          <t>Uzaklık: +%-8.08</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3495,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>269.75</v>
+        <v>268.33</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -3407,7 +3520,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>295.79</v>
+        <v>295.5</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -3432,7 +3545,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>26.6</v>
+        <v>26.3</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -3441,7 +3554,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BIST 100 Dolar bazında 224.35$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.7) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.7 aşağıda, 52 haftalık dibinden (223.54$) ise %0.4 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.79$) altında baskı altında seyrederken RSI(14) göstergesi 26.6 seviyesindedir.</t>
+          <t>BIST 100 Dolar bazında 223.99$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.4) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.8 aşağıda, 52 haftalık dibinden (223.54$) ise %0.2 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.5$) altında baskı altında seyrederken RSI(14) göstergesi 26.3 seviyesindedir.</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5635,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>27/100 (Korku)</t>
+          <t>33/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5657,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>28/100 (Korku)</t>
+          <t>33/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5679,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>50/100 (Nötr)</t>
+          <t>48/100 (Nötr)</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5696,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın faizi %36'ya indirme kararı nasıl yorumlandı?</t>
+          <t>Merkez Bankası'nın 9 ay sonra ilk kez faiz indirmesi ne anlama geliyor?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -5666,17 +5779,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Euronews.com</t>
+          <t>Anadolu Ajansı</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TCMB faiz kararını açıkladı: Ocaktan bu yana ilk faiz indirimi</t>
+          <t>Üç büyük merkez bankası enflasyon riskleri altında faiz kararı alacak</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>TCMB, Faiz</t>
+          <t>Merkez Bankası, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -5688,17 +5801,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Anadolu Ajansı</t>
+          <t>DW.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Üç büyük merkez bankası enflasyon riskleri altında faiz kararı alacak</t>
+          <t>Merkez Bankası'nın faiz indirimi işe yarayacak mı?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz, Enflasyon</t>
+          <t>Merkez Bankası, Faiz</t>
         </is>
       </c>
     </row>
@@ -5710,17 +5823,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Habertürk</t>
+          <t>Bloomberght</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan, Türkiye'deki bankacılık faaliyetlerini büyütme kararı aldığını açıkladı</t>
+          <t>Fitch: Türkiye'nin borçlanma piyasası 2027'ye kadar 550 milyar dolara ulaşabilir</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan</t>
+          <t>Fitch</t>
         </is>
       </c>
     </row>
@@ -5732,17 +5845,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Uzmanpara</t>
+          <t>Habertürk</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>GÖZLER FED'İN FAİZ KARARINA ÇEVRİLDİ! FED toplantısı ne zaman, faiz kararı hangi gün saat kaçta açıklanacak? Amerikan Merkez Bankası (FED) Ekim ayı faiz beklentisi ne yönde?</t>
+          <t>JPMorgan, Türkiye'deki bankacılık faaliyetlerini büyütme kararı aldığını açıkladı</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Fed, Faiz</t>
+          <t>JPMorgan</t>
         </is>
       </c>
     </row>
@@ -5754,17 +5867,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CNBC-e</t>
+          <t>Euronews.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>ECB faiz kararı öncesi 5 kritik soru: Piyasalar ne bekliyor?</t>
+          <t>Enflasyon ve petrol fiyatları Fed'in faiz kararını nasıl etkileyecek?</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ECB, Faiz</t>
+          <t>Fed, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -5776,17 +5889,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Platin Dergisi</t>
+          <t>Uzmanpara</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Fed faiz kararı ne zaman? Beklentiler ne yönde?</t>
+          <t>GÖZLER FED'İN FAİZ KARARINA ÇEVRİLDİ! FED toplantısı ne zaman, faiz kararı hangi gün saat kaçta açıklanacak? Amerikan Merkez Bankası (FED) Ekim ayı faiz beklentisi ne yönde?</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Fed, Faiz</t>
+          <t>Merkez Bankası, Fed, Faiz</t>
         </is>
       </c>
     </row>
@@ -5820,12 +5933,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Son Dakika</t>
+          <t>Akdenizmanset</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>TÜİK'e göre Uşak'ta Eylül'de satılan konut sayısı 52 artışla 770'e ulaştı</t>
+          <t>TÜİK eylül ayı konut satış rakamlarını açıkladı</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
📊 Otomatik Günlük Finans Raporu ve Excel Güncellemesi (2026-10-28)
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI5"/>
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1166,6 +1166,119 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>11165.44</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>224.05</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>-32.81</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>295.21</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>7743.98</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>4077.4</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>6532.86</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>54.11</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>75.34999999999999</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>49.83</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>55.57</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="S6" s="2" t="n">
+        <v>102.14</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="U6" s="2" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="V6" s="2" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="W6" s="2" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="X6" s="2" t="n">
+        <v>81139.63</v>
+      </c>
+      <c r="Y6" s="2" t="n">
+        <v>2353.55</v>
+      </c>
+      <c r="Z6" s="2" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="AA6" s="2" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="AB6" s="2" t="n">
+        <v>59.48</v>
+      </c>
+      <c r="AC6" s="2" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="AD6" s="2" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="AE6" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="AF6" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="AG6" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>TI2 (%2.42)</t>
+        </is>
+      </c>
+      <c r="AI6" s="2" t="inlineStr">
+        <is>
+          <t>IIH (%74.5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1273,41 +1386,41 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>11151.03</v>
+        <v>11165.44</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>-0.01% (Yatay)</t>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>+0.13% (Artış)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>-5.48% (Azalış)</t>
+          <t>-3.56% (Azalış)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>-11.45% (Azalış)</t>
+          <t>-9.15% (Azalış)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>-16.11% (Azalış)</t>
+          <t>-17.04% (Azalış)</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>-0.98% (Azalış)</t>
+          <t>-0.85% (Azalış)</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>+2.74% (Artış)</t>
+          <t>+2.71% (Artış)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -1333,41 +1446,41 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13934.73</v>
+        <v>13960.89</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>-0.10% (Yatay)</t>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>+0.19% (Artış)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>-5.05% (Azalış)</t>
+          <t>-3.48% (Azalış)</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>-10.95% (Azalış)</t>
+          <t>-8.54% (Azalış)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>-7.31% (Azalış)</t>
+          <t>-8.44% (Azalış)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>+14.00% (Artış)</t>
+          <t>+14.21% (Artış)</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>+17.48% (Artış)</t>
+          <t>+17.50% (Artış)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -1393,7 +1506,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>15313.58</v>
+        <v>15068.21</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -1402,32 +1515,32 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>-0.60% (Azalış)</t>
+          <t>-1.60% (Azalış)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>-5.17% (Azalış)</t>
+          <t>-5.39% (Azalış)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>-5.02% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>+4.97% (Artış)</t>
+          <t>-6.64% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>+0.39% (Yatay)</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>-7.41% (Azalış)</t>
+          <t>-8.90% (Azalış)</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>+6.08% (Artış)</t>
+          <t>+4.57% (Artış)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1453,41 +1566,41 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13656.29</v>
+        <v>13600.8</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>+0.54% (Artış)</t>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>-0.41% (Azalış)</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>-6.73% (Azalış)</t>
+          <t>-4.48% (Azalış)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>-17.76% (Azalış)</t>
+          <t>-15.57% (Azalış)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>-25.65% (Azalış)</t>
+          <t>-26.39% (Azalış)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>-2.55% (Azalış)</t>
+          <t>-2.94% (Azalış)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>-3.11% (Azalış)</t>
+          <t>-3.52% (Azalış)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1513,7 +1626,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7722.6</v>
+        <v>7743.98</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -1522,32 +1635,32 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>+0.60% (Artış)</t>
+          <t>+0.28% (Artış)</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>+0.13% (Yatay)</t>
+          <t>-0.17% (Yatay)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>+0.51% (Artış)</t>
+          <t>+0.95% (Artış)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>+5.56% (Artış)</t>
+          <t>+4.12% (Artış)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>+12.81% (Artış)</t>
+          <t>+13.13% (Artış)</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>+12.07% (Artış)</t>
+          <t>+12.38% (Artış)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1573,7 +1686,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>26477.81</v>
+        <v>26549.85</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -1582,32 +1695,32 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>+1.18% (Artış)</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>+0.20% (Yatay)</t>
+          <t>+0.27% (Artış)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>-0.57% (Azalış)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>-1.28% (Azalış)</t>
+          <t>-0.92% (Azalış)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>+8.32% (Artış)</t>
+          <t>+5.68% (Artış)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>+13.92% (Artış)</t>
+          <t>+14.23% (Artış)</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>+11.12% (Artış)</t>
+          <t>+10.82% (Artış)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1633,41 +1746,41 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>52377.57</v>
+        <v>52475.1</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>+0.03% (Yatay)</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>-0.23% (Yatay)</t>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>+0.19% (Artış)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>-0.72% (Azalış)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>+1.74% (Artış)</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>+1.52% (Artış)</t>
+          <t>+2.19% (Artış)</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>+0.51% (Yatay)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>+8.98% (Artış)</t>
+          <t>+9.18% (Artış)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>+9.79% (Artış)</t>
+          <t>+10.17% (Artış)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1693,7 +1806,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>17.57</v>
+        <v>16.91</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -1702,32 +1815,32 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>-4.46% (Azalış)</t>
+          <t>-3.48% (Azalış)</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>+1.50% (Artış)</t>
+          <t>+1.38% (Artış)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>+9.33% (Artış)</t>
+          <t>+5.42% (Artış)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>+2.81% (Artış)</t>
+          <t>+5.75% (Artış)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>+17.53% (Artış)</t>
+          <t>+13.11% (Artış)</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>+11.27% (Artış)</t>
+          <t>+2.98% (Artış)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1753,41 +1866,41 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>4072.7</v>
+        <v>4077.4</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>+0.85% (Artış)</t>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>+0.07% (Yatay)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>-1.69% (Azalış)</t>
+          <t>-1.75% (Azalış)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>-2.30% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>+0.90% (Artış)</t>
+          <t>-2.45% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>-0.55% (Yatay)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>-6.18% (Azalış)</t>
+          <t>-6.07% (Azalış)</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>+1.32% (Artış)</t>
+          <t>+2.37% (Artış)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1813,41 +1926,41 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>54.46</v>
+        <v>54.11</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>+0.65% (Artış)</t>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>-0.34% (Azalış)</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>-5.63% (Azalış)</t>
+          <t>-5.77% (Azalış)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-11.04% (Azalış)</t>
+          <t>-10.81% (Azalış)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>-5.88% (Azalış)</t>
+          <t>-8.00% (Azalış)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>-22.35% (Azalış)</t>
+          <t>-22.85% (Azalış)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+16.96% (Artış)</t>
+          <t>+14.82% (Artış)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1873,7 +1986,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>80666.64999999999</v>
+        <v>81139.63</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1882,32 +1995,32 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>+0.82% (Artış)</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>-0.79% (Azalış)</t>
+          <t>+0.41% (Artış)</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>+0.08% (Yatay)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-5.72% (Azalış)</t>
+          <t>-2.57% (Azalış)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>+2.68% (Artış)</t>
+          <t>+2.67% (Artış)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-7.82% (Azalış)</t>
+          <t>-7.28% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-29.31% (Azalış)</t>
+          <t>-28.17% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1933,7 +2046,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2343.52</v>
+        <v>2353.55</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -1942,32 +2055,32 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>+1.00% (Artış)</t>
+          <t>+0.25% (Artış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-1.79% (Azalış)</t>
+          <t>-1.28% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-13.12% (Azalış)</t>
+          <t>-8.55% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-4.08% (Azalış)</t>
+          <t>-6.09% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-21.01% (Azalış)</t>
+          <t>-20.68% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-43.12% (Azalış)</t>
+          <t>-40.90% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1993,41 +2106,41 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>+1.19% (Artış)</t>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>-0.28% (Azalış)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>+1.14% (Artış)</t>
+          <t>+2.47% (Artış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-11.68% (Azalış)</t>
+          <t>-6.71% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-7.73% (Azalış)</t>
+          <t>-6.79% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-28.12% (Azalış)</t>
+          <t>-27.94% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-49.80% (Azalış)</t>
+          <t>-49.12% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -2053,41 +2166,41 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>49.78</v>
+        <v>49.83</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>+0.09% (Yatay)</t>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>+0.11% (Artış)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>+0.43% (Artış)</t>
+          <t>+0.50% (Artış)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>+1.66% (Artış)</t>
+          <t>+1.71% (Artış)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>+5.09% (Artış)</t>
+          <t>+4.91% (Artış)</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>+15.90% (Artış)</t>
+          <t>+16.02% (Artış)</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+18.55% (Artış)</t>
+          <t>+18.77% (Artış)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -2113,7 +2226,7 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55.48</v>
+        <v>55.57</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -2122,32 +2235,32 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>-0.63% (Azalış)</t>
+          <t>-0.14% (Azalış)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>-0.23% (Yatay)</t>
+          <t>-0.22% (Yatay)</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>-0.46% (Yatay)</t>
+          <t>-0.31% (Yatay)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>+1.99% (Artış)</t>
+          <t>+1.56% (Artış)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>+9.64% (Artış)</t>
+          <t>+9.81% (Artış)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>+13.49% (Artış)</t>
+          <t>+13.71% (Artış)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -2173,7 +2286,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1.11</v>
+        <v>1.12</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -2182,27 +2295,27 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>-0.73% (Azalış)</t>
+          <t>-0.16% (Azalış)</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>-0.71% (Azalış)</t>
+          <t>-0.63% (Azalış)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-2.13% (Azalış)</t>
+          <t>-1.91% (Azalış)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>-2.89% (Azalış)</t>
+          <t>-3.19% (Azalış)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>-5.20% (Azalış)</t>
+          <t>-5.04% (Azalış)</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -2233,41 +2346,41 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>102.33</v>
+        <v>102.14</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>+0.36% (Artış)</t>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>-0.18% (Azalış)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>+0.58% (Artış)</t>
+          <t>+0.35% (Artış)</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>+1.11% (Artış)</t>
+          <t>+0.76% (Artış)</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>+1.51% (Artış)</t>
+          <t>+2.13% (Artış)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>+4.12% (Artış)</t>
+          <t>+3.93% (Artış)</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>+3.59% (Artış)</t>
+          <t>+3.49% (Artış)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2293,7 +2406,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>4.84</v>
+        <v>4.87</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -2302,32 +2415,32 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>+0.33% (Artış)</t>
+          <t>+0.64% (Artış)</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>-1.93% (Azalış)</t>
+          <t>-2.03% (Azalış)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>-4.50% (Azalış)</t>
+          <t>-3.79% (Azalış)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>+11.21% (Artış)</t>
+          <t>+11.34% (Artış)</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>+30.04% (Artış)</t>
+          <t>+30.87% (Artış)</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>+33.92% (Artış)</t>
+          <t>+34.82% (Artış)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -2353,7 +2466,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>4.99</v>
+        <v>5.04</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -2362,32 +2475,32 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>+0.14% (Artış)</t>
+          <t>+1.04% (Artış)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>-2.42% (Azalış)</t>
+          <t>-1.96% (Azalış)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>-4.71% (Azalış)</t>
+          <t>-4.00% (Azalış)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>+8.03% (Artış)</t>
+          <t>+8.19% (Artış)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>+19.94% (Artış)</t>
+          <t>+21.19% (Artış)</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>+24.92% (Artış)</t>
+          <t>+26.66% (Artış)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2413,41 +2526,41 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>5.3</v>
+        <v>5.36</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>+0.08% (Yatay)</t>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>+1.06% (Artış)</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>-2.21% (Azalış)</t>
+          <t>-1.43% (Azalış)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>-4.60% (Azalış)</t>
+          <t>-4.17% (Azalış)</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>+3.15% (Artış)</t>
+          <t>+2.94% (Artış)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>+9.61% (Artış)</t>
+          <t>+10.76% (Artış)</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>+16.08% (Artış)</t>
+          <t>+17.90% (Artış)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2653,7 +2766,7 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>109.84</v>
+        <v>110.3</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -2662,32 +2775,32 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>-5.15% (Azalış)</t>
+          <t>-3.14% (Azalış)</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>+0.97% (Artış)</t>
+          <t>+1.36% (Artış)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>+4.33% (Artış)</t>
+          <t>+7.52% (Artış)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>+21.05% (Artış)</t>
+          <t>+23.89% (Artış)</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>+80.51% (Artış)</t>
+          <t>+81.27% (Artış)</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>+67.39% (Artış)</t>
+          <t>+71.27% (Artış)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2713,7 +2826,7 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>6.66</v>
+        <v>6.68</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -2722,32 +2835,32 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>+2.28% (Artış)</t>
+          <t>+0.91% (Artış)</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>+1.37% (Artış)</t>
+          <t>+2.13% (Artış)</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>+1.38% (Artış)</t>
+          <t>+2.12% (Artış)</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>+6.11% (Artış)</t>
+          <t>+3.69% (Artış)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>+18.23% (Artış)</t>
+          <t>+18.69% (Artış)</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>+29.49% (Artış)</t>
+          <t>+30.00% (Artış)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2773,7 +2886,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>611</v>
+        <v>599.5</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -2782,32 +2895,32 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>-0.81% (Azalış)</t>
+          <t>-1.76% (Azalış)</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>-5.01% (Azalış)</t>
+          <t>-4.58% (Azalış)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-11.29% (Azalış)</t>
+          <t>-13.46% (Azalış)</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>-7.53% (Azalış)</t>
+          <t>-9.65% (Azalış)</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>+20.51% (Artış)</t>
+          <t>+18.24% (Artış)</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>+16.16% (Artış)</t>
+          <t>+13.33% (Artış)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2833,7 +2946,7 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>294.25</v>
+        <v>286.35</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -2842,32 +2955,32 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>-2.23% (Azalış)</t>
+          <t>-2.52% (Azalış)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>-5.48% (Azalış)</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>+1.90% (Artış)</t>
+          <t>-9.43% (Azalış)</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>-1.07% (Azalış)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>-9.68% (Azalış)</t>
+          <t>-11.36% (Azalış)</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>-15.63% (Azalış)</t>
+          <t>-17.89% (Azalış)</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>-24.57% (Azalış)</t>
+          <t>-26.18% (Azalış)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -2893,7 +3006,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>6518.54</v>
+        <v>6532.86</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -2902,7 +3015,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>+0.94% (Artış)</t>
+          <t>+0.18% (Artış)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2953,7 +3066,7 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>74.78</v>
+        <v>75.34999999999999</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -2962,17 +3075,17 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>+0.19% (Artış)</t>
+          <t>+0.40% (Artış)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>+4.16% (Artış)</t>
+          <t>+4.26% (Artış)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>+9.83% (Artış)</t>
+          <t>+9.38% (Artış)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2982,17 +3095,17 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>+20.81% (Artış)</t>
+          <t>+21.73% (Artış)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>-13.38% (Azalış)</t>
+          <t>-10.85% (Azalış)</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Altın/Gümüş oranı 74.78 ile dengeli bantta seyrediyor.</t>
+          <t>Altın/Gümüş oranı 75.35 ile dengeli bantta seyrediyor.</t>
         </is>
       </c>
     </row>
@@ -3056,11 +3169,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>223.99</v>
+        <v>224.05</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TL: 11151.03 / Kur: 49.78</t>
+          <t>TL: 11165.44 / Kur: 49.83</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3082,7 +3195,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>%-0.1</t>
+          <t>%0.02</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -3109,7 +3222,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>%-5.86</t>
+          <t>%-3.96</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3136,7 +3249,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>%-12.85</t>
+          <t>%-10.66</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3163,7 +3276,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>%-19.96</t>
+          <t>%-20.92</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -3190,7 +3303,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>%-14.57</t>
+          <t>%-14.55</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -3217,7 +3330,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>%-13.34</t>
+          <t>%-13.52</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3252,7 +3365,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Zirveden %-32.82 aşağıda</t>
+          <t>Zirveden %-32.81 aşağıda</t>
         </is>
       </c>
     </row>
@@ -3277,7 +3390,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dipten +%0.2 yukarıda</t>
+          <t>Dipten +%0.23 yukarıda</t>
         </is>
       </c>
     </row>
@@ -3294,7 +3407,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>%0.4</t>
+          <t>%0.5</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3329,7 +3442,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tavana uzaklık: %-26.58</t>
+          <t>Tavana uzaklık: %-26.56</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3467,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Tabandan uzaklık: +%0.2</t>
+          <t>Tabandan uzaklık: +%0.23</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3492,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: %-25.13</t>
+          <t>Uzaklık: %-25.11</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3517,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: +%-8.08</t>
+          <t>Uzaklık: +%-8.06</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3608,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>268.33</v>
+        <v>266.78</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -3520,7 +3633,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>295.5</v>
+        <v>295.21</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -3554,7 +3667,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BIST 100 Dolar bazında 223.99$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.4) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.8 aşağıda, 52 haftalık dibinden (223.54$) ise %0.2 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.5$) altında baskı altında seyrederken RSI(14) göstergesi 26.3 seviyesindedir.</t>
+          <t>BIST 100 Dolar bazında 224.05$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.5) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.8 aşağıda, 52 haftalık dibinden (223.54$) ise %0.2 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.21$) altında baskı altında seyrederken RSI(14) göstergesi 26.3 seviyesindedir.</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -5061,22 +5174,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Bugün Açıklananlar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TCMB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -5086,7 +5199,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
+          <t>Fed Faiz Kararı</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -5096,19 +5209,19 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4.00%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Bugün Açıklananlar</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -5133,7 +5246,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Fed Faiz Kararı</t>
+          <t>Fed (FOMC) Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -5143,19 +5256,19 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Bugün Açıklananlar</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -5165,7 +5278,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -5180,7 +5293,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Fed (FOMC) Para Politikası Açıklaması</t>
+          <t>Fed Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -5207,7 +5320,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -5217,7 +5330,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Türkiye (TCMB)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -5227,7 +5340,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Fed Başkanı Basın Toplantısı</t>
+          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -5254,17 +5367,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-03</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Türkiye (TÜİK)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -5274,7 +5387,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Öncü GSYH Büyüme Oranı (Çeyreklik)</t>
+          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -5284,12 +5397,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5434,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Çekirdek PCE Enflasyon Endeksi (Aylık)</t>
+          <t>Öncü GSYH Büyüme Oranı (Çeyreklik)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -5331,12 +5444,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>1.5%</t>
         </is>
       </c>
     </row>
@@ -5353,12 +5466,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -5368,7 +5481,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Avrupa Merkez Bankası (ECB) Faiz Kararı</t>
+          <t>Çekirdek PCE Enflasyon Endeksi (Aylık)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5378,12 +5491,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>0.3%</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>0.2%</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5528,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>ECB Para Politikası Açıklaması</t>
+          <t>Avrupa Merkez Bankası (ECB) Faiz Kararı</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5425,12 +5538,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.65%</t>
         </is>
       </c>
     </row>
@@ -5447,7 +5560,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -5462,7 +5575,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ECB Başkanı Basın Toplantısı</t>
+          <t>ECB Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -5484,22 +5597,22 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Gelecek Hafta Açıklanacaklar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -5509,7 +5622,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
+          <t>ECB Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5570,6 +5683,53 @@
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Gelecek Hafta Açıklanacaklar</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-10</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Türkiye (TÜİK)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Yüksek</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>TÜİK Sanayi Üretim Endeksi ve İşgücü İstatistikleri</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5635,7 +5795,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>33/100 (Korku)</t>
+          <t>36/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5657,7 +5817,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>33/100 (Korku)</t>
+          <t>34/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5839,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>48/100 (Nötr)</t>
+          <t>51/100 (Nötr)</t>
         </is>
       </c>
     </row>
@@ -5696,7 +5856,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın 9 ay sonra ilk kez faiz indirmesi ne anlama geliyor?</t>
+          <t>Merkez Bankası'nın faizi %36'ya indirme kararı nasıl yorumlandı?</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -5735,12 +5895,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Investing.com Türkiye</t>
+          <t>Euronews.com</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TCMB Faiz Kararını Bugün Açıklıyor: Beklentiler ve Piyasa Senaryoları</t>
+          <t>TCMB faiz kararını açıkladı: Ocaktan bu yana ilk faiz indirimi</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -5779,17 +5939,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Anadolu Ajansı</t>
+          <t>DW.com</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Üç büyük merkez bankası enflasyon riskleri altında faiz kararı alacak</t>
+          <t>Merkez Bankası'nın faiz indirimi işe yarayacak mı?</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz, Enflasyon</t>
+          <t>Merkez Bankası, Faiz</t>
         </is>
       </c>
     </row>
@@ -5801,17 +5961,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DW.com</t>
+          <t>Anadolu Ajansı</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın faiz indirimi işe yarayacak mı?</t>
+          <t>Üç büyük merkez bankası enflasyon riskleri altında faiz kararı alacak</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz</t>
+          <t>Merkez Bankası, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -5845,17 +6005,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Habertürk</t>
+          <t>Anadolu Ajansı</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan, Türkiye'deki bankacılık faaliyetlerini büyütme kararı aldığını açıkladı</t>
+          <t>Fitch Ratings, Türkiye'de borçlanma sermaye piyasasının büyümeye devam edeceğini öngörüyor</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan</t>
+          <t>Fitch</t>
         </is>
       </c>
     </row>
@@ -5867,17 +6027,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Euronews.com</t>
+          <t>Foreks.com</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Enflasyon ve petrol fiyatları Fed'in faiz kararını nasıl etkileyecek?</t>
+          <t>SPK başvurusu JPMorgan Chase grubunun Türkiye'den çekilmesi anlamına gelmiyor</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Fed, Faiz, Enflasyon</t>
+          <t>JPMorgan, SPK</t>
         </is>
       </c>
     </row>
@@ -5889,17 +6049,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Uzmanpara</t>
+          <t>CNN Türk</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>GÖZLER FED'İN FAİZ KARARINA ÇEVRİLDİ! FED toplantısı ne zaman, faiz kararı hangi gün saat kaçta açıklanacak? Amerikan Merkez Bankası (FED) Ekim ayı faiz beklentisi ne yönde?</t>
+          <t>Fitch'ten Türkiye için olumlu tahmin! 550 milyar dolara ulaşacak</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Fed, Faiz</t>
+          <t>Fitch</t>
         </is>
       </c>
     </row>
@@ -5933,12 +6093,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Akdenizmanset</t>
+          <t>Anadolu Ajansı</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>TÜİK eylül ayı konut satış rakamlarını açıkladı</t>
+          <t>Türkiye'de eylülde 142 bin 390 konut satıldı</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
📊 Otomatik Günlük Finans Raporu ve Excel Güncellemesi (2026-10-29)
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI6"/>
+  <dimension ref="A1:AI7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1279,6 +1279,119 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>11165.4</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>224.21</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>-32.76</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>295.21</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>7720.39</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>4037.3</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>6468.42</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>52.31</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>83.81</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>77.18000000000001</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>49.83</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>55.81</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="S7" s="2" t="n">
+        <v>101.91</v>
+      </c>
+      <c r="T7" s="2" t="n">
+        <v>4.99</v>
+      </c>
+      <c r="U7" s="2" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="V7" s="2" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="W7" s="2" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="X7" s="2" t="n">
+        <v>80346.41</v>
+      </c>
+      <c r="Y7" s="2" t="n">
+        <v>2317.62</v>
+      </c>
+      <c r="Z7" s="2" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="AA7" s="2" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="AB7" s="2" t="n">
+        <v>59.52</v>
+      </c>
+      <c r="AC7" s="2" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="AD7" s="2" t="n">
+        <v>6.59</v>
+      </c>
+      <c r="AE7" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="AF7" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="AG7" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="AH7" s="2" t="inlineStr">
+        <is>
+          <t>TI2 (%2.42)</t>
+        </is>
+      </c>
+      <c r="AI7" s="2" t="inlineStr">
+        <is>
+          <t>IIH (%74.5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1386,7 +1499,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>11165.44</v>
+        <v>11165.4</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -1446,7 +1559,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13960.89</v>
+        <v>13960.9</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -1506,7 +1619,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>15068.21</v>
+        <v>15068.2</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -1626,41 +1739,41 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7743.98</v>
+        <v>7720.39</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>+0.28% (Artış)</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>-0.17% (Yatay)</t>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>-0.30% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>+0.74% (Artış)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>+0.95% (Artış)</t>
+          <t>+0.90% (Artış)</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>+4.12% (Artış)</t>
+          <t>+3.08% (Artış)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>+13.13% (Artış)</t>
+          <t>+12.78% (Artış)</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>+12.38% (Artış)</t>
+          <t>+13.16% (Artış)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1686,41 +1799,41 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>26549.85</v>
+        <v>26184.72</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>+0.27% (Artış)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>-0.57% (Azalış)</t>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>-1.38% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>+0.68% (Artış)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>-0.92% (Azalış)</t>
+          <t>-2.52% (Azalış)</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>+5.68% (Artış)</t>
+          <t>+3.20% (Artış)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>+14.23% (Artış)</t>
+          <t>+12.66% (Artış)</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>+10.82% (Artış)</t>
+          <t>+11.04% (Artış)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1746,41 +1859,41 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>52475.1</v>
+        <v>52342.56</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>+0.19% (Artış)</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>-0.25% (Azalış)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>-0.72% (Azalış)</t>
+          <t>-0.99% (Azalış)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>+2.19% (Artış)</t>
+          <t>+2.82% (Artış)</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>+0.51% (Yatay)</t>
+          <t>-0.27% (Yatay)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>+9.18% (Artış)</t>
+          <t>+8.90% (Artış)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>+10.17% (Artış)</t>
+          <t>+10.14% (Artış)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1806,41 +1919,41 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>16.91</v>
+        <v>17.2</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>-3.48% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>+1.38% (Artış)</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>+1.71% (Artış)</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>-9.62% (Azalış)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>+5.42% (Artış)</t>
+          <t>+5.26% (Artış)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>+5.75% (Artış)</t>
+          <t>+8.45% (Artış)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>+13.11% (Artış)</t>
+          <t>+15.05% (Artış)</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>+2.98% (Artış)</t>
+          <t>+1.65% (Artış)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1866,41 +1979,41 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>4077.4</v>
+        <v>4037.3</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>+0.07% (Yatay)</t>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>-0.35% (Azalış)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>-1.75% (Azalış)</t>
+          <t>-0.57% (Azalış)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>-2.45% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>-0.55% (Yatay)</t>
+          <t>-3.57% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>-1.70% (Azalış)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>-6.07% (Azalış)</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>+2.37% (Artış)</t>
+          <t>-7.00% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>+0.91% (Yatay)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1926,7 +2039,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>54.11</v>
+        <v>52.31</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -1935,32 +2048,32 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>-0.34% (Azalış)</t>
+          <t>-2.15% (Azalış)</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>-5.77% (Azalış)</t>
+          <t>-4.48% (Azalış)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-10.81% (Azalış)</t>
+          <t>-12.96% (Azalış)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>-8.00% (Azalış)</t>
+          <t>-9.17% (Azalış)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>-22.85% (Azalış)</t>
+          <t>-25.41% (Azalış)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+14.82% (Artış)</t>
+          <t>+9.62% (Artış)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -1986,41 +2099,41 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>81139.63</v>
+        <v>80346.41</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>+0.41% (Artış)</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>+0.08% (Yatay)</t>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>-1.13% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>-0.55% (Azalış)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-2.57% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>+2.67% (Artış)</t>
+          <t>-1.63% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>+0.11% (Yatay)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-7.28% (Azalış)</t>
+          <t>-8.18% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-28.17% (Azalış)</t>
+          <t>-26.99% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -2046,41 +2159,41 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2353.55</v>
+        <v>2317.62</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>+0.25% (Artış)</t>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>-1.70% (Azalış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-1.28% (Azalış)</t>
+          <t>-1.63% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-8.55% (Azalış)</t>
+          <t>-6.24% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-6.09% (Azalış)</t>
+          <t>-7.68% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-20.68% (Azalış)</t>
+          <t>-21.89% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-40.90% (Azalış)</t>
+          <t>-40.62% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -2106,7 +2219,7 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1.33</v>
+        <v>1.27</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
@@ -2115,32 +2228,32 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>-0.28% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>+2.47% (Artış)</t>
+          <t>-4.08% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>-2.17% (Azalış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-6.71% (Azalış)</t>
+          <t>-7.88% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-6.79% (Azalış)</t>
+          <t>-12.58% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-27.94% (Azalış)</t>
+          <t>-30.96% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-49.12% (Azalış)</t>
+          <t>-50.22% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -2173,24 +2286,24 @@
           <t>TL</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>+0.11% (Artış)</t>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>+0.07% (Yatay)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>+0.50% (Artış)</t>
+          <t>+0.42% (Artış)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>+1.71% (Artış)</t>
+          <t>+1.68% (Artış)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>+4.91% (Artış)</t>
+          <t>+4.84% (Artış)</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -2200,7 +2313,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+18.77% (Artış)</t>
+          <t>+18.80% (Artış)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -2226,41 +2339,41 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55.57</v>
+        <v>55.81</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>-0.14% (Azalış)</t>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>+0.65% (Artış)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>-0.22% (Yatay)</t>
+          <t>+0.10% (Yatay)</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>-0.31% (Yatay)</t>
+          <t>+0.35% (Yatay)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>+1.56% (Artış)</t>
+          <t>+1.67% (Artış)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>+9.81% (Artış)</t>
+          <t>+10.29% (Artış)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>+13.71% (Artış)</t>
+          <t>+14.01% (Artış)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -2293,34 +2406,34 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>-0.16% (Azalış)</t>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>+0.47% (Artış)</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>-0.63% (Azalış)</t>
+          <t>-0.47% (Azalış)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-1.91% (Azalış)</t>
+          <t>-1.40% (Azalış)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>-3.19% (Azalış)</t>
+          <t>-3.14% (Azalış)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>-5.04% (Azalış)</t>
+          <t>-4.81% (Azalış)</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>-4.26% (Azalış)</t>
+          <t>-4.08% (Azalış)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2346,7 +2459,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>102.14</v>
+        <v>101.91</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -2355,32 +2468,32 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>-0.18% (Azalış)</t>
+          <t>-0.27% (Azalış)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>+0.35% (Artış)</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>+0.76% (Artış)</t>
+          <t>+0.30% (Artış)</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>+0.45% (Yatay)</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>+2.13% (Artış)</t>
+          <t>+2.12% (Artış)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>+3.93% (Artış)</t>
+          <t>+3.69% (Artış)</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>+3.49% (Artış)</t>
+          <t>+2.71% (Artış)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2406,41 +2519,41 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>4.87</v>
+        <v>4.8</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>+0.64% (Artış)</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>-2.03% (Azalış)</t>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>-1.44% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>+0.69% (Artış)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>-3.79% (Azalış)</t>
+          <t>-5.66% (Azalış)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>+11.34% (Artış)</t>
+          <t>+7.65% (Artış)</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>+30.87% (Artış)</t>
+          <t>+28.99% (Artış)</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>+34.82% (Artış)</t>
+          <t>+29.86% (Artış)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -2466,41 +2579,41 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>5.04</v>
+        <v>4.99</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>+1.04% (Artış)</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>-1.96% (Azalış)</t>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>-1.11% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>+0.73% (Artış)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>-4.00% (Azalış)</t>
+          <t>-5.74% (Azalış)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>+8.19% (Artış)</t>
+          <t>+5.14% (Artış)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>+21.19% (Artış)</t>
+          <t>+19.84% (Artış)</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>+26.66% (Artış)</t>
+          <t>+22.94% (Artış)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2526,41 +2639,41 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>5.36</v>
+        <v>5.33</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>+1.06% (Artış)</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>-1.43% (Azalış)</t>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>-0.60% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>+0.79% (Artış)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>-4.17% (Azalış)</t>
+          <t>-5.48% (Azalış)</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>+2.94% (Artış)</t>
+          <t>+1.02% (Artış)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>+10.76% (Artış)</t>
+          <t>+10.10% (Artış)</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>+17.90% (Artış)</t>
+          <t>+15.85% (Artış)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2766,7 +2879,7 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>110.3</v>
+        <v>111.7</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -2778,29 +2891,29 @@
           <t>-3.14% (Azalış)</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>+1.36% (Artış)</t>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>-1.30% (Azalış)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>+7.52% (Artış)</t>
+          <t>+7.89% (Artış)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>+23.89% (Artış)</t>
+          <t>+23.95% (Artış)</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>+81.27% (Artış)</t>
+          <t>+83.57% (Artış)</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>+71.27% (Artış)</t>
+          <t>+72.06% (Artış)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2826,41 +2939,41 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>6.68</v>
+        <v>6.59</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>+0.91% (Artış)</t>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>-0.72% (Azalış)</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>+2.13% (Artış)</t>
+          <t>+3.64% (Artış)</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>+2.12% (Artış)</t>
+          <t>+0.53% (Artış)</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>+3.69% (Artış)</t>
+          <t>+2.45% (Artış)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>+18.69% (Artış)</t>
+          <t>+17.12% (Artış)</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>+30.00% (Artış)</t>
+          <t>+26.00% (Artış)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2886,41 +2999,41 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>599.5</v>
+        <v>603.25</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>cent</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>-1.76% (Azalış)</t>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>+0.71% (Artış)</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>-4.58% (Azalış)</t>
+          <t>-3.44% (Azalış)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-13.46% (Azalış)</t>
+          <t>-10.73% (Azalış)</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>-9.65% (Azalış)</t>
+          <t>-5.63% (Azalış)</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>+18.24% (Artış)</t>
+          <t>+18.98% (Artış)</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>+13.33% (Artış)</t>
+          <t>+13.34% (Artış)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -2946,41 +3059,41 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>286.35</v>
+        <v>286.55</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>cent</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>-2.52% (Azalış)</t>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>-0.07% (Yatay)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>-9.43% (Azalış)</t>
+          <t>-8.29% (Azalış)</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>-1.07% (Azalış)</t>
+          <t>-1.43% (Azalış)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>-11.36% (Azalış)</t>
+          <t>-13.72% (Azalış)</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>-17.89% (Azalış)</t>
+          <t>-17.84% (Azalış)</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>-26.18% (Azalış)</t>
+          <t>-26.66% (Azalış)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -3006,16 +3119,16 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>6532.86</v>
+        <v>6468.42</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>+0.18% (Artış)</t>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>-0.29% (Azalış)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3066,7 +3179,7 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>75.34999999999999</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -3075,17 +3188,17 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>+0.40% (Artış)</t>
+          <t>+1.83% (Artış)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>+4.26% (Artış)</t>
+          <t>+4.10% (Artış)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>+9.38% (Artış)</t>
+          <t>+10.80% (Artış)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -3095,17 +3208,17 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>+21.73% (Artış)</t>
+          <t>+24.68% (Artış)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>-10.85% (Azalış)</t>
+          <t>-7.94% (Azalış)</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Altın/Gümüş oranı 75.35 ile dengeli bantta seyrediyor.</t>
+          <t>Altın/Gümüş oranı 77.18 ile dengeli bantta seyrediyor.</t>
         </is>
       </c>
     </row>
@@ -3169,11 +3282,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>224.05</v>
+        <v>224.21</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TL: 11165.44 / Kur: 49.83</t>
+          <t>TL: 11165.4 / Kur: 49.83</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3195,7 +3308,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>%0.02</t>
+          <t>%0.09</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -3222,7 +3335,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>%-3.96</t>
+          <t>%-3.9</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3249,7 +3362,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>%-10.66</t>
+          <t>%-10.6</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3276,7 +3389,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>%-20.92</t>
+          <t>%-20.86</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -3303,7 +3416,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>%-14.55</t>
+          <t>%-14.49</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -3330,7 +3443,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>%-13.52</t>
+          <t>%-13.48</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3365,7 +3478,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Zirveden %-32.81 aşağıda</t>
+          <t>Zirveden %-32.76 aşağıda</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3503,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dipten +%0.23 yukarıda</t>
+          <t>Dipten +%0.3 yukarıda</t>
         </is>
       </c>
     </row>
@@ -3407,7 +3520,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>%0.5</t>
+          <t>%0.6</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3442,7 +3555,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tavana uzaklık: %-26.56</t>
+          <t>Tavana uzaklık: %-26.51</t>
         </is>
       </c>
     </row>
@@ -3467,7 +3580,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Tabandan uzaklık: +%0.23</t>
+          <t>Tabandan uzaklık: +%0.3</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3605,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: %-25.11</t>
+          <t>Uzaklık: %-25.05</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3630,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: +%-8.06</t>
+          <t>Uzaklık: +%-7.99</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3771,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>26.3</v>
+        <v>26.6</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -3667,7 +3780,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BIST 100 Dolar bazında 224.05$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.5) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.8 aşağıda, 52 haftalık dibinden (223.54$) ise %0.2 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.21$) altında baskı altında seyrederken RSI(14) göstergesi 26.3 seviyesindedir.</t>
+          <t>BIST 100 Dolar bazında 224.21$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.6) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.8 aşağıda, 52 haftalık dibinden (223.54$) ise %0.3 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.21$) altında baskı altında seyrederken RSI(14) göstergesi 26.6 seviyesindedir.</t>
         </is>
       </c>
     </row>
@@ -5179,17 +5292,17 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Türkiye (TCMB)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -5199,7 +5312,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Fed Faiz Kararı</t>
+          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -5209,12 +5322,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5226,12 +5339,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -5246,7 +5359,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Fed (FOMC) Para Politikası Açıklaması</t>
+          <t>Öncü GSYH Büyüme Oranı (Çeyreklik)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -5256,12 +5369,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.5%</t>
         </is>
       </c>
     </row>
@@ -5273,12 +5386,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -5293,7 +5406,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Fed Başkanı Basın Toplantısı</t>
+          <t>Çekirdek PCE Enflasyon Endeksi (Aylık)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -5303,19 +5416,19 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.3%</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.2%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Bugün Açıklananlar</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -5325,12 +5438,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TCMB)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -5340,7 +5453,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
+          <t>Avrupa Merkez Bankası (ECB) Faiz Kararı</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -5350,34 +5463,34 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2.65%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Bugün Açıklananlar</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -5387,7 +5500,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
+          <t>ECB Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -5409,7 +5522,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Bu Hafta Açıklanacaklar</t>
+          <t>Bugün Açıklananlar</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -5419,12 +5532,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -5434,7 +5547,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Öncü GSYH Büyüme Oranı (Çeyreklik)</t>
+          <t>ECB Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -5444,12 +5557,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5461,17 +5574,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-03</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Türkiye (TÜİK)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -5481,7 +5594,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Çekirdek PCE Enflasyon Endeksi (Aylık)</t>
+          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5491,12 +5604,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -5508,17 +5621,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -5528,7 +5641,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Avrupa Merkez Bankası (ECB) Faiz Kararı</t>
+          <t>Fed Faiz Kararı</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5538,12 +5651,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>4.00%</t>
         </is>
       </c>
     </row>
@@ -5555,17 +5668,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -5575,7 +5688,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>ECB Para Politikası Açıklaması</t>
+          <t>Fed (FOMC) Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -5602,17 +5715,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -5622,7 +5735,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>ECB Başkanı Basın Toplantısı</t>
+          <t>Fed Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5795,7 +5908,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>36/100 (Korku)</t>
+          <t>35/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5930,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>34/100 (Korku)</t>
+          <t>31/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5851,17 +5964,17 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>BBC</t>
+          <t>Anadolu Ajansı</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın faizi %36'ya indirme kararı nasıl yorumlandı?</t>
+          <t>Üç büyük merkez bankası enflasyon riskleri altında faiz kararı alacak</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz</t>
+          <t>Merkez Bankası, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -5873,17 +5986,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>TRT Haber</t>
+          <t>Gazete Oksijen</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası faiz kararını açıkladı</t>
+          <t>Üç büyük merkez bankası için kritik hafta: Enflasyon faiz kararlarını nasıl etkileyecek?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz</t>
+          <t>Merkez Bankası, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -5895,17 +6008,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Euronews.com</t>
+          <t>Investing.com Türkiye</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>TCMB faiz kararını açıkladı: Ocaktan bu yana ilk faiz indirimi</t>
+          <t>Kanada Merkez Bankası enflasyon endişesiyle üç yılın ilk faiz artışını yaptı</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>TCMB, Faiz</t>
+          <t>Merkez Bankası, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -5917,12 +6030,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Uzmanpara</t>
+          <t>Dünya Gazetesi</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Son dakika...Merkez Bankası faiz kararını açıklayacak! İşte piyasanın tahmini</t>
+          <t>Merkez Bankası'nın faiz kararının ardından 16 kurumdan yeni tahmin</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -5939,12 +6052,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DW.com</t>
+          <t>İstanbul Ticaret Gazetesi</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın faiz indirimi işe yarayacak mı?</t>
+          <t>Kanada Merkez Bankası faiz kararını açıkladı: 2023’ten sonra ilk artış</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -5961,17 +6074,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Anadolu Ajansı</t>
+          <t>Ekonomim</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Üç büyük merkez bankası enflasyon riskleri altında faiz kararı alacak</t>
+          <t>Goldman Sachs'tan TCMB'nin faiz kararına uyarı: Rezerv kaybı riski</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz, Enflasyon</t>
+          <t>TCMB, Faiz, Goldman Sachs</t>
         </is>
       </c>
     </row>
@@ -6027,17 +6140,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Foreks.com</t>
+          <t>Ekonomim</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>SPK başvurusu JPMorgan Chase grubunun Türkiye'den çekilmesi anlamına gelmiyor</t>
+          <t>Fitch'ten Türkiye tahmini: Borçlanma piyasasında büyüme beklentisi 550 milyar dolar</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>JPMorgan, SPK</t>
+          <t>Fitch</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Otomatik Günlük Finans Raporu ve Excel Güncellemesi (2026-10-30)
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI7"/>
+  <dimension ref="A1:AI8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1392,6 +1392,119 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>10759.56</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>-3.63</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>215.43</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>-35.39</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>294.86</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>7566.48</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>-1.99</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>3886.1</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>6240.12</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>49.02</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>78.70999999999999</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>79.28</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>55.81</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="S8" s="2" t="n">
+        <v>101.91</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="U8" s="2" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="V8" s="2" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="W8" s="2" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="X8" s="2" t="n">
+        <v>76806.31</v>
+      </c>
+      <c r="Y8" s="2" t="n">
+        <v>2236.01</v>
+      </c>
+      <c r="Z8" s="2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="AA8" s="2" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="AB8" s="2" t="n">
+        <v>59.04</v>
+      </c>
+      <c r="AC8" s="2" t="n">
+        <v>112.61</v>
+      </c>
+      <c r="AD8" s="2" t="n">
+        <v>6.48</v>
+      </c>
+      <c r="AE8" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="AF8" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="AG8" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH8" s="2" t="inlineStr">
+        <is>
+          <t>TI2 (%2.42)</t>
+        </is>
+      </c>
+      <c r="AI8" s="2" t="inlineStr">
+        <is>
+          <t>IIH (%74.5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1499,41 +1612,41 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>11165.4</v>
+        <v>10759.56</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>+0.13% (Artış)</t>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>-3.63% (Azalış)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>-3.56% (Azalış)</t>
+          <t>-4.11% (Azalış)</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>-9.15% (Azalış)</t>
+          <t>-9.94% (Azalış)</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>-17.04% (Azalış)</t>
+          <t>-19.77% (Azalış)</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>-0.85% (Azalış)</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>+2.71% (Artış)</t>
+          <t>-4.46% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
+        <is>
+          <t>-0.72% (Yatay)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -1559,41 +1672,41 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13960.9</v>
+        <v>13419.68</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>puan</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>+0.19% (Artış)</t>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>-3.88% (Azalış)</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>-3.48% (Azalış)</t>
+          <t>-4.22% (Azalış)</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>-8.54% (Azalış)</t>
+          <t>-9.58% (Azalış)</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>-8.44% (Azalış)</t>
+          <t>-11.74% (Azalış)</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>+14.21% (Artış)</t>
+          <t>+9.79% (Artış)</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>+17.50% (Artış)</t>
+          <t>+13.72% (Artış)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -1619,7 +1732,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>15068.2</v>
+        <v>14607.53</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -1628,32 +1741,32 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>-1.60% (Azalış)</t>
+          <t>-3.06% (Azalış)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>-5.39% (Azalış)</t>
+          <t>-4.84% (Azalış)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>-6.64% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>+0.39% (Yatay)</t>
+          <t>-5.15% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>-5.51% (Azalış)</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>-8.90% (Azalış)</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>+4.57% (Artış)</t>
+          <t>-11.68% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>+0.75% (Yatay)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1679,7 +1792,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>13600.8</v>
+        <v>12982.61</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -1688,32 +1801,32 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>-0.41% (Azalış)</t>
+          <t>-4.55% (Azalış)</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>-4.48% (Azalış)</t>
+          <t>-5.89% (Azalış)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>-15.57% (Azalış)</t>
+          <t>-16.82% (Azalış)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>-26.39% (Azalış)</t>
+          <t>-28.98% (Azalış)</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>-2.94% (Azalış)</t>
+          <t>-7.35% (Azalış)</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>-3.52% (Azalış)</t>
+          <t>-8.50% (Azalış)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -1739,7 +1852,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7720.39</v>
+        <v>7566.48</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -1748,32 +1861,32 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>-0.30% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>+0.74% (Artış)</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>+0.90% (Artış)</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>+3.08% (Artış)</t>
+          <t>-1.99% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>-0.75% (Azalış)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>-1.30% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>-0.45% (Yatay)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>+12.78% (Artış)</t>
+          <t>+10.53% (Artış)</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>+13.16% (Artış)</t>
+          <t>+10.62% (Artış)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1799,7 +1912,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>26184.72</v>
+        <v>25422.07</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -1808,32 +1921,32 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>-1.38% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>+0.68% (Artış)</t>
+          <t>-2.91% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>-2.05% (Azalış)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>-2.52% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>+3.20% (Artış)</t>
+          <t>-5.39% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>-1.90% (Azalış)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>+12.66% (Artış)</t>
+          <t>+9.38% (Artış)</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>+11.04% (Artış)</t>
+          <t>+7.15% (Artış)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1859,7 +1972,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>52342.56</v>
+        <v>51787.51</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -1868,32 +1981,32 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>-0.25% (Azalış)</t>
+          <t>-1.06% (Azalış)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>-0.99% (Azalış)</t>
+          <t>-0.82% (Azalış)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>+2.82% (Artış)</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>-0.27% (Yatay)</t>
+          <t>+1.69% (Artış)</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>-2.62% (Azalış)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>+8.90% (Artış)</t>
+          <t>+7.75% (Artış)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>+10.14% (Artış)</t>
+          <t>+8.88% (Artış)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -1919,7 +2032,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>17.2</v>
+        <v>21.16</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -1928,32 +2041,32 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>+1.71% (Artış)</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>-9.62% (Azalış)</t>
+          <t>+23.02% (Artış)</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>+8.79% (Artış)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>+5.26% (Artış)</t>
+          <t>+29.10% (Artış)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>+8.45% (Artış)</t>
+          <t>+28.24% (Artış)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>+15.05% (Artış)</t>
+          <t>+41.54% (Artış)</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>+1.65% (Artış)</t>
+          <t>+25.13% (Artış)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1979,7 +2092,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>4037.3</v>
+        <v>3886.1</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -1988,32 +2101,32 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>-0.35% (Azalış)</t>
+          <t>-3.60% (Azalış)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>-0.57% (Azalış)</t>
+          <t>-3.04% (Azalış)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>-3.57% (Azalış)</t>
+          <t>-7.52% (Azalış)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>-1.70% (Azalış)</t>
+          <t>-5.00% (Azalış)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>-7.00% (Azalış)</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>+0.91% (Yatay)</t>
+          <t>-10.48% (Azalış)</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>-3.23% (Azalış)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -2039,7 +2152,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>52.31</v>
+        <v>49.02</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -2048,32 +2161,32 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>-2.15% (Azalış)</t>
+          <t>-6.08% (Azalış)</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>-4.48% (Azalış)</t>
+          <t>-8.73% (Azalış)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-12.96% (Azalış)</t>
+          <t>-19.28% (Azalış)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>-9.17% (Azalış)</t>
+          <t>-14.99% (Azalış)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>-25.41% (Azalış)</t>
+          <t>-30.11% (Azalış)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+9.62% (Artış)</t>
+          <t>+1.22% (Artış)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -2099,7 +2212,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>80346.41</v>
+        <v>76806.31</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -2108,32 +2221,32 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>-1.13% (Azalış)</t>
+          <t>-1.25% (Azalış)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>-0.55% (Azalış)</t>
+          <t>-4.02% (Azalış)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-1.63% (Azalış)</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>+0.11% (Yatay)</t>
+          <t>-6.95% (Azalış)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>-1.32% (Azalış)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-8.18% (Azalış)</t>
+          <t>-12.23% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-26.99% (Azalış)</t>
+          <t>-29.08% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -2159,7 +2272,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2317.62</v>
+        <v>2236.01</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
@@ -2168,32 +2281,32 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>-1.70% (Azalış)</t>
+          <t>-0.60% (Azalış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-1.63% (Azalış)</t>
+          <t>-3.91% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-6.24% (Azalış)</t>
+          <t>-10.04% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-7.68% (Azalış)</t>
+          <t>-8.46% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-21.89% (Azalış)</t>
+          <t>-24.64% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-40.62% (Azalış)</t>
+          <t>-41.23% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -2219,41 +2332,41 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>1.27</v>
+        <v>1.25</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>-4.08% (Azalış)</t>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>+0.92% (Artış)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>-2.17% (Azalış)</t>
+          <t>-3.72% (Azalış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-7.88% (Azalış)</t>
+          <t>-10.69% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-12.58% (Azalış)</t>
+          <t>-9.90% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-30.96% (Azalış)</t>
+          <t>-32.27% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-50.22% (Azalış)</t>
+          <t>-48.92% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -2279,41 +2392,41 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>49.83</v>
+        <v>49.94</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
           <t>TL</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>+0.07% (Yatay)</t>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>+0.23% (Artış)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>+0.42% (Artış)</t>
+          <t>+0.43% (Artış)</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>+1.68% (Artış)</t>
+          <t>+1.87% (Artış)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>+4.84% (Artış)</t>
+          <t>+5.06% (Artış)</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>+16.02% (Artış)</t>
+          <t>+16.28% (Artış)</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+18.80% (Artış)</t>
+          <t>+19.21% (Artış)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -2348,32 +2461,32 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>+0.65% (Artış)</t>
+          <t>+0.23% (Artış)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>+0.10% (Yatay)</t>
+          <t>-0.06% (Yatay)</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>+0.35% (Yatay)</t>
+          <t>+0.47% (Yatay)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>+1.67% (Artış)</t>
+          <t>+2.00% (Artış)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>+10.29% (Artış)</t>
+          <t>+10.30% (Artış)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>+14.01% (Artış)</t>
+          <t>+14.54% (Artış)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -2408,32 +2521,32 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>+0.47% (Artış)</t>
+          <t>+0.13% (Artış)</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>-0.47% (Azalış)</t>
+          <t>-0.45% (Azalış)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-1.40% (Azalış)</t>
+          <t>-1.38% (Azalış)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>-3.14% (Azalış)</t>
+          <t>-2.93% (Azalış)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>-4.81% (Azalış)</t>
+          <t>-4.91% (Azalış)</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>-4.08% (Azalış)</t>
+          <t>-3.73% (Azalış)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2468,22 +2581,22 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>-0.27% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>+0.30% (Artış)</t>
+          <t>-0.13% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>+0.10% (Yatay)</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>+0.45% (Yatay)</t>
+          <t>-0.19% (Yatay)</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>+2.12% (Artış)</t>
+          <t>+1.95% (Artış)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -2493,7 +2606,7 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>+2.71% (Artış)</t>
+          <t>+2.39% (Artış)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2519,7 +2632,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>4.8</v>
+        <v>4.72</v>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
@@ -2528,32 +2641,32 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>-1.44% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>+0.69% (Artış)</t>
+          <t>-1.67% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>-1.75% (Azalış)</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>-5.66% (Azalış)</t>
+          <t>-5.67% (Azalış)</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>+7.65% (Artış)</t>
+          <t>+7.30% (Artış)</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>+28.99% (Artış)</t>
+          <t>+26.84% (Artış)</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>+29.86% (Artış)</t>
+          <t>+26.91% (Artış)</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -2579,7 +2692,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>4.99</v>
+        <v>4.92</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -2588,32 +2701,32 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>-1.11% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>+0.73% (Artış)</t>
+          <t>-1.40% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>-1.38% (Azalış)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>-5.74% (Azalış)</t>
+          <t>-6.07% (Azalış)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>+5.14% (Artış)</t>
+          <t>+4.97% (Artış)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>+19.84% (Artış)</t>
+          <t>+18.16% (Artış)</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>+22.94% (Artış)</t>
+          <t>+20.18% (Artış)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2639,7 +2752,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>5.33</v>
+        <v>5.3</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -2648,32 +2761,32 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>-0.60% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>+0.79% (Artış)</t>
+          <t>-0.45% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>-0.19% (Yatay)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>-5.48% (Azalış)</t>
+          <t>-5.32% (Azalış)</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>+1.02% (Artış)</t>
+          <t>+1.41% (Artış)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>+10.10% (Artış)</t>
+          <t>+9.61% (Artış)</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>+15.85% (Artış)</t>
+          <t>+14.16% (Artış)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2879,7 +2992,7 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>111.7</v>
+        <v>112.61</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
@@ -2888,32 +3001,32 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>-3.14% (Azalış)</t>
+          <t>-1.98% (Azalış)</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>-1.30% (Azalış)</t>
+          <t>-3.52% (Azalış)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>+7.89% (Artış)</t>
+          <t>+10.07% (Artış)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>+23.95% (Artış)</t>
+          <t>+34.43% (Artış)</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>+83.57% (Artış)</t>
+          <t>+85.06% (Artış)</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>+72.06% (Artış)</t>
+          <t>+73.25% (Artış)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2939,7 +3052,7 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>6.59</v>
+        <v>6.48</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -2948,32 +3061,32 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>-0.72% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>+3.64% (Artış)</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>+0.53% (Artış)</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>+2.45% (Artış)</t>
+          <t>-1.57% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>+0.02% (Yatay)</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>-0.07% (Yatay)</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>-0.56% (Yatay)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>+17.12% (Artış)</t>
+          <t>+15.05% (Artış)</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>+26.00% (Artış)</t>
+          <t>+27.56% (Artış)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -3006,24 +3119,24 @@
           <t>cent</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>+0.71% (Artış)</t>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>-0.08% (Yatay)</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>-3.44% (Azalış)</t>
+          <t>-3.48% (Azalış)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-10.73% (Azalış)</t>
+          <t>-11.64% (Azalış)</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>-5.63% (Azalış)</t>
+          <t>-7.33% (Azalış)</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
@@ -3033,7 +3146,7 @@
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>+13.34% (Artış)</t>
+          <t>+15.07% (Artış)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -3059,41 +3172,41 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>286.55</v>
+        <v>287.15</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>cent</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>-0.07% (Yatay)</t>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>+0.60% (Artış)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>-8.29% (Azalış)</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>-1.43% (Azalış)</t>
+          <t>-6.60% (Azalış)</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>-0.38% (Yatay)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>-13.72% (Azalış)</t>
+          <t>-10.13% (Azalış)</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>-17.84% (Azalış)</t>
+          <t>-17.66% (Azalış)</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>-26.66% (Azalış)</t>
+          <t>-26.75% (Azalış)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -3119,7 +3232,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>6468.42</v>
+        <v>6240.12</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -3128,7 +3241,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>-0.29% (Azalış)</t>
+          <t>-3.38% (Azalış)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3179,7 +3292,7 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>77.18000000000001</v>
+        <v>79.28</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -3188,17 +3301,17 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>+1.83% (Artış)</t>
+          <t>+2.64% (Artış)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>+4.10% (Artış)</t>
+          <t>+6.24% (Artış)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>+10.80% (Artış)</t>
+          <t>+14.57% (Artış)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -3208,17 +3321,17 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>+24.68% (Artış)</t>
+          <t>+28.08% (Artış)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>-7.94% (Azalış)</t>
+          <t>-4.40% (Azalış)</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Altın/Gümüş oranı 77.18 ile dengeli bantta seyrediyor.</t>
+          <t>Altın/Gümüş oranı 79.28 ile dengeli bantta seyrediyor.</t>
         </is>
       </c>
     </row>
@@ -3282,11 +3395,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>224.21</v>
+        <v>215.43</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TL: 11165.4 / Kur: 49.83</t>
+          <t>TL: 10759.56 / Kur: 49.94</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3308,7 +3421,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>%0.09</t>
+          <t>%-3.92</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -3318,7 +3431,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Yatay</t>
+          <t>Azalış</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3448,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>%-3.9</t>
+          <t>%-4.52</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3362,7 +3475,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>%-10.6</t>
+          <t>%-11.59</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3389,7 +3502,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>%-20.86</t>
+          <t>%-23.63</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -3416,7 +3529,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>%-14.49</t>
+          <t>%-17.83</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -3443,7 +3556,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>%-13.48</t>
+          <t>%-16.71</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3478,7 +3591,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Zirveden %-32.76 aşağıda</t>
+          <t>Zirveden %-35.39 aşağıda</t>
         </is>
       </c>
     </row>
@@ -3494,16 +3607,16 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>223.54</v>
+        <v>215.43</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dipten +%0.3 yukarıda</t>
+          <t>Dipten +%0.0 yukarıda</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3633,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>%0.6</t>
+          <t>%0.0</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3555,7 +3668,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Tavana uzaklık: %-26.51</t>
+          <t>Tavana uzaklık: %-29.38</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3684,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>223.54</v>
+        <v>215.43</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -3580,7 +3693,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Tabandan uzaklık: +%0.3</t>
+          <t>Tabandan uzaklık: +%0.0</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3718,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: %-25.05</t>
+          <t>Uzaklık: %-27.99</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3743,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Uzaklık: +%-7.99</t>
+          <t>Uzaklık: +%-11.59</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3759,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>265.52</v>
+        <v>260.51</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -3671,7 +3784,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>278.49</v>
+        <v>274.44</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -3696,7 +3809,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>291.46</v>
+        <v>288.36</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -3721,7 +3834,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>266.78</v>
+        <v>265.1</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -3746,7 +3859,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>295.21</v>
+        <v>294.86</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -3771,7 +3884,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>26.6</v>
+        <v>22.2</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -3780,7 +3893,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BIST 100 Dolar bazında 224.21$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.6) yer alıyor. 52 haftalık zirvesinden (333.44$) %32.8 aşağıda, 52 haftalık dibinden (223.54$) ise %0.3 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (295.21$) altında baskı altında seyrederken RSI(14) göstergesi 26.6 seviyesindedir.</t>
+          <t>BIST 100 Dolar bazında 215.43$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.0) yer alıyor. 52 haftalık zirvesinden (333.44$) %35.4 aşağıda, 52 haftalık dibinden (215.43$) ise %0.0 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (294.86$) altında baskı altında seyrederken RSI(14) göstergesi 22.2 seviyesindedir.</t>
         </is>
       </c>
     </row>
@@ -5287,22 +5400,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bugün Açıklananlar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-03</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TCMB)</t>
+          <t>Türkiye (TÜİK)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -5312,7 +5425,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
+          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -5334,22 +5447,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Bugün Açıklananlar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Türkiye (TCMB)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -5359,7 +5472,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Öncü GSYH Büyüme Oranı (Çeyreklik)</t>
+          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -5369,29 +5482,29 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>3.2%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>1.5%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Bugün Açıklananlar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -5406,7 +5519,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Çekirdek PCE Enflasyon Endeksi (Aylık)</t>
+          <t>Fed Faiz Kararı</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -5416,34 +5529,34 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>0.3%</t>
+          <t>4.00%</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>0.2%</t>
+          <t>4.00%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Bugün Açıklananlar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -5453,7 +5566,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Avrupa Merkez Bankası (ECB) Faiz Kararı</t>
+          <t>Fed (FOMC) Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -5463,34 +5576,34 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2.65%</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bugün Açıklananlar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -5500,7 +5613,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>ECB Para Politikası Açıklaması</t>
+          <t>Fed Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -5522,7 +5635,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Bugün Açıklananlar</t>
+          <t>Bu Hafta Açıklanacaklar</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -5532,12 +5645,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Euro Bölgesi (ECB)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -5547,7 +5660,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>ECB Başkanı Basın Toplantısı</t>
+          <t>Öncü GSYH Büyüme Oranı (Çeyreklik)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -5557,12 +5670,12 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>3.2%</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.5%</t>
         </is>
       </c>
     </row>
@@ -5574,17 +5687,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>2026-11-03</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>ABD (Fed/Makro)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -5594,7 +5707,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Aylık ve Yıllık TÜFE (Enflasyon) Verileri</t>
+          <t>Çekirdek PCE Enflasyon Endeksi (Aylık)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5604,12 +5717,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.3%</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0.2%</t>
         </is>
       </c>
     </row>
@@ -5621,17 +5734,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -5641,7 +5754,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Fed Faiz Kararı</t>
+          <t>Avrupa Merkez Bankası (ECB) Faiz Kararı</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5651,12 +5764,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>2.65%</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>4.00%</t>
+          <t>2.65%</t>
         </is>
       </c>
     </row>
@@ -5668,17 +5781,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -5688,7 +5801,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Fed (FOMC) Para Politikası Açıklaması</t>
+          <t>ECB Para Politikası Açıklaması</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -5715,17 +5828,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ABD (Fed/Makro)</t>
+          <t>Euro Bölgesi (ECB)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -5735,7 +5848,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Fed Başkanı Basın Toplantısı</t>
+          <t>ECB Başkanı Basın Toplantısı</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5762,17 +5875,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TCMB)</t>
+          <t>Türkiye (TÜİK)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -5782,7 +5895,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
+          <t>TÜİK Sanayi Üretim Endeksi ve İşgücü İstatistikleri</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -5809,17 +5922,17 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Türkiye (TÜİK)</t>
+          <t>Türkiye (TCMB)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -5829,7 +5942,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>TÜİK Sanayi Üretim Endeksi ve İşgücü İstatistikleri</t>
+          <t>TCMB Haftalık Uluslararası Rezervler ve Yabancı Menkul Kıymet İstatistikleri</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -5908,7 +6021,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>35/100 (Korku)</t>
+          <t>24/100 (Aşırı Korku)</t>
         </is>
       </c>
     </row>
@@ -5930,7 +6043,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>31/100 (Korku)</t>
+          <t>21/100 (Aşırı Korku)</t>
         </is>
       </c>
     </row>
@@ -5952,7 +6065,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>51/100 (Nötr)</t>
+          <t>30/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -5986,12 +6099,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Gazete Oksijen</t>
+          <t>Investing.com Türkiye</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Üç büyük merkez bankası için kritik hafta: Enflasyon faiz kararlarını nasıl etkileyecek?</t>
+          <t>Goldman, Çek Merkez Bankası faiz görüşünü enflasyon riskleri nedeniyle yükseltti</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -6008,12 +6121,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Investing.com Türkiye</t>
+          <t>Gazete Oksijen</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Kanada Merkez Bankası enflasyon endişesiyle üç yılın ilk faiz artışını yaptı</t>
+          <t>Üç büyük merkez bankası için kritik hafta: Enflasyon faiz kararlarını nasıl etkileyecek?</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6030,17 +6143,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Dünya Gazetesi</t>
+          <t>Foreks.com</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası'nın faiz kararının ardından 16 kurumdan yeni tahmin</t>
+          <t>Japonya Merkez Bankası faizi yüzde 1,25'te tuttu, enflasyon tahminlerini yükseltti</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz</t>
+          <t>Merkez Bankası, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -6074,17 +6187,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Ekonomim</t>
+          <t>Euronews.com</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs'tan TCMB'nin faiz kararına uyarı: Rezerv kaybı riski</t>
+          <t>Enflasyon ve petrol fiyatları Fed'in faiz kararını nasıl etkileyecek?</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>TCMB, Faiz, Goldman Sachs</t>
+          <t>Fed, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -6206,12 +6319,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Anadolu Ajansı</t>
+          <t>Bloomberght</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Türkiye'de eylülde 142 bin 390 konut satıldı</t>
+          <t>Konut satışları Eylül'de yıllık düşüş serisini sürdürdü</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
📊 Otomatik Günlük Finans Raporu ve Excel Güncellemesi (2026-10-31)
</commit_message>
<xml_diff>
--- a/docs/Finans_Veri_Tabani.xlsx
+++ b/docs/Finans_Veri_Tabani.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI8"/>
+  <dimension ref="A1:AI9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1505,6 +1505,119 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>10759.6</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>-3.63</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>215.44</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>-35.39</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>294.86</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>7580.07</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>-1.82</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>3898.9</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>6260.46</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>78.83</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>79.41</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>49.94</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>55.86</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="S9" s="2" t="n">
+        <v>101.88</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>4.93</v>
+      </c>
+      <c r="U9" s="2" t="n">
+        <v>38.45</v>
+      </c>
+      <c r="V9" s="2" t="n">
+        <v>28.15</v>
+      </c>
+      <c r="W9" s="2" t="n">
+        <v>258.4</v>
+      </c>
+      <c r="X9" s="2" t="n">
+        <v>77431.66</v>
+      </c>
+      <c r="Y9" s="2" t="n">
+        <v>2250.46</v>
+      </c>
+      <c r="Z9" s="2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="AA9" s="2" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="AB9" s="2" t="n">
+        <v>59.24</v>
+      </c>
+      <c r="AC9" s="2" t="n">
+        <v>117.64</v>
+      </c>
+      <c r="AD9" s="2" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="AE9" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="AF9" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="AG9" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="AH9" s="2" t="inlineStr">
+        <is>
+          <t>TI2 (%2.42)</t>
+        </is>
+      </c>
+      <c r="AI9" s="2" t="inlineStr">
+        <is>
+          <t>IIH (%74.5)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1612,7 +1725,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>10759.56</v>
+        <v>10759.6</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -1672,7 +1785,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>13419.68</v>
+        <v>13419.7</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -1732,7 +1845,7 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>14607.53</v>
+        <v>14607.5</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -1766,7 +1879,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>+0.75% (Yatay)</t>
+          <t>+0.74% (Yatay)</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -1792,7 +1905,7 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>12982.61</v>
+        <v>12982.6</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -1852,7 +1965,7 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>7566.48</v>
+        <v>7580.07</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -1861,32 +1974,32 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>-1.99% (Azalış)</t>
+          <t>-1.82% (Azalış)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>-0.75% (Azalış)</t>
+          <t>-0.57% (Azalış)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>-1.30% (Azalış)</t>
+          <t>-1.13% (Azalış)</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>-0.45% (Yatay)</t>
+          <t>-0.27% (Yatay)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>+10.53% (Artış)</t>
+          <t>+10.73% (Artış)</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>+10.62% (Artış)</t>
+          <t>+10.82% (Artış)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1912,7 +2025,7 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>25422.07</v>
+        <v>25437</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -1921,32 +2034,32 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>-2.91% (Azalış)</t>
+          <t>-2.86% (Azalış)</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>-2.05% (Azalış)</t>
+          <t>-2.00% (Azalış)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>-5.39% (Azalış)</t>
+          <t>-5.34% (Azalış)</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>-1.90% (Azalış)</t>
+          <t>-1.84% (Azalış)</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>+9.38% (Artış)</t>
+          <t>+9.44% (Artış)</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>+7.15% (Artış)</t>
+          <t>+7.22% (Artış)</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1972,7 +2085,7 @@
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>51787.51</v>
+        <v>51770.31</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -1981,32 +2094,32 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>-1.06% (Azalış)</t>
+          <t>-1.09% (Azalış)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>-0.82% (Azalış)</t>
+          <t>-0.85% (Azalış)</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>+1.69% (Artış)</t>
+          <t>+1.66% (Artış)</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>-2.62% (Azalış)</t>
+          <t>-2.65% (Azalış)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>+7.75% (Artış)</t>
+          <t>+7.71% (Artış)</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>+8.88% (Artış)</t>
+          <t>+8.85% (Artış)</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -2032,7 +2145,7 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>21.16</v>
+        <v>19.42</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -2041,32 +2154,32 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>+23.02% (Artış)</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>+8.79% (Artış)</t>
+          <t>+12.91% (Artış)</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>-0.15% (Yatay)</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>+29.10% (Artış)</t>
+          <t>+18.49% (Artış)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>+28.24% (Artış)</t>
+          <t>+17.70% (Artış)</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>+41.54% (Artış)</t>
+          <t>+29.90% (Artış)</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>+25.13% (Artış)</t>
+          <t>+14.84% (Artış)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -2092,7 +2205,7 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>3886.1</v>
+        <v>3898.9</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -2101,32 +2214,32 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>-3.60% (Azalış)</t>
+          <t>-3.29% (Azalış)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>-3.04% (Azalış)</t>
+          <t>-2.72% (Azalış)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>-7.52% (Azalış)</t>
+          <t>-7.22% (Azalış)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>-5.00% (Azalış)</t>
+          <t>-4.68% (Azalış)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>-10.48% (Azalış)</t>
+          <t>-10.19% (Azalış)</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>-3.23% (Azalış)</t>
+          <t>-2.44% (Azalış)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -2152,7 +2265,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>49.02</v>
+        <v>49.1</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -2161,32 +2274,32 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>-6.08% (Azalış)</t>
+          <t>-5.93% (Azalış)</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>-8.73% (Azalış)</t>
+          <t>-8.59% (Azalış)</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>-19.28% (Azalış)</t>
+          <t>-19.15% (Azalış)</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>-14.99% (Azalış)</t>
+          <t>-14.86% (Azalış)</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>-30.11% (Azalış)</t>
+          <t>-30.00% (Azalış)</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>+1.22% (Artış)</t>
+          <t>+2.30% (Artış)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -2212,41 +2325,41 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>76806.31</v>
+        <v>77431.66</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>-1.25% (Azalış)</t>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>+0.30% (Artış)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>-4.02% (Azalış)</t>
+          <t>-3.22% (Azalış)</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>-6.95% (Azalış)</t>
+          <t>-6.61% (Azalış)</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>-1.32% (Azalış)</t>
+          <t>-1.04% (Azalış)</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>-12.23% (Azalış)</t>
+          <t>-11.52% (Azalış)</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>-29.08% (Azalış)</t>
+          <t>-29.32% (Azalış)</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -2272,41 +2385,41 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>2236.01</v>
+        <v>2250.46</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>-0.60% (Azalış)</t>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>+0.42% (Artış)</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>-3.91% (Azalış)</t>
+          <t>-3.01% (Azalış)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>-10.04% (Azalış)</t>
+          <t>-10.13% (Azalış)</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>-8.46% (Azalış)</t>
+          <t>-8.43% (Azalış)</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-24.64% (Azalış)</t>
+          <t>-24.15% (Azalış)</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>-41.23% (Azalış)</t>
+          <t>-41.50% (Azalış)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -2339,34 +2452,34 @@
           <t>USD</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>+0.92% (Artış)</t>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>-0.17% (Azalış)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>-3.72% (Azalış)</t>
+          <t>-4.18% (Azalış)</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>-10.69% (Azalış)</t>
+          <t>-10.66% (Azalış)</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>-9.90% (Azalış)</t>
+          <t>-10.34% (Azalış)</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>-32.27% (Azalış)</t>
+          <t>-31.94% (Azalış)</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>-48.92% (Azalış)</t>
+          <t>-50.08% (Azalış)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -2416,7 +2529,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>+5.06% (Artış)</t>
+          <t>+5.05% (Artış)</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -2426,7 +2539,7 @@
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>+19.21% (Artış)</t>
+          <t>+19.20% (Artış)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -2452,7 +2565,7 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>55.81</v>
+        <v>55.86</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
@@ -2461,32 +2574,32 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>+0.23% (Artış)</t>
+          <t>+0.30% (Artış)</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>-0.06% (Yatay)</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>+0.47% (Yatay)</t>
+          <t>+0.01% (Yatay)</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>+0.55% (Artış)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>+2.00% (Artış)</t>
+          <t>+2.08% (Artış)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>+10.30% (Artış)</t>
+          <t>+10.39% (Artış)</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>+14.54% (Artış)</t>
+          <t>+14.63% (Artış)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -2521,32 +2634,32 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>+0.13% (Artış)</t>
+          <t>+0.24% (Artış)</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>-0.45% (Azalış)</t>
+          <t>-0.34% (Azalış)</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>-1.38% (Azalış)</t>
+          <t>-1.27% (Azalış)</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>-2.93% (Azalış)</t>
+          <t>-2.82% (Azalış)</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>-4.91% (Azalış)</t>
+          <t>-4.81% (Azalış)</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
         <is>
-          <t>-3.73% (Azalış)</t>
+          <t>-3.62% (Azalış)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -2572,7 +2685,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>101.91</v>
+        <v>101.88</v>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
@@ -2581,32 +2694,32 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>-0.13% (Azalış)</t>
+          <t>-0.16% (Azalış)</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>+0.10% (Yatay)</t>
+          <t>+0.07% (Yatay)</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>-0.19% (Yatay)</t>
+          <t>-0.22% (Yatay)</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>+1.95% (Artış)</t>
+          <t>+1.92% (Artış)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>+3.69% (Artış)</t>
+          <t>+3.66% (Artış)</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>+2.39% (Artış)</t>
+          <t>+2.08% (Artış)</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -2692,7 +2805,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>4.92</v>
+        <v>4.93</v>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
@@ -2701,32 +2814,32 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>-1.40% (Azalış)</t>
+          <t>-1.20% (Azalış)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>-1.38% (Azalış)</t>
+          <t>-1.18% (Azalış)</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>-6.07% (Azalış)</t>
+          <t>-5.88% (Azalış)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>+4.97% (Artış)</t>
+          <t>+5.19% (Artış)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>+18.16% (Artış)</t>
+          <t>+18.40% (Artış)</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>+20.18% (Artış)</t>
+          <t>+20.43% (Artış)</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -2752,7 +2865,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>5.3</v>
+        <v>5.31</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
@@ -2761,32 +2874,32 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>-0.45% (Azalış)</t>
+          <t>-0.38% (Azalış)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>-0.19% (Yatay)</t>
+          <t>-0.11% (Yatay)</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>-5.32% (Azalış)</t>
+          <t>-5.25% (Azalış)</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>+1.41% (Artış)</t>
+          <t>+1.49% (Artış)</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>+9.61% (Artış)</t>
+          <t>+9.69% (Artış)</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>+14.16% (Artış)</t>
+          <t>+14.25% (Artış)</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2992,41 +3105,41 @@
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>112.61</v>
+        <v>117.64</v>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>-1.98% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>-3.52% (Azalış)</t>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>+2.40% (Artış)</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>+0.79% (Artış)</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>+10.07% (Artış)</t>
+          <t>+14.98% (Artış)</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>+34.43% (Artış)</t>
+          <t>+40.43% (Artış)</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>+85.06% (Artış)</t>
+          <t>+93.33% (Artış)</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>+73.25% (Artış)</t>
+          <t>+80.79% (Artış)</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -3052,7 +3165,7 @@
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>6.48</v>
+        <v>6.46</v>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
@@ -3061,32 +3174,32 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>-1.57% (Azalış)</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>+0.02% (Yatay)</t>
+          <t>-1.86% (Azalış)</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>-0.27% (Azalış)</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>-0.07% (Yatay)</t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>-0.56% (Yatay)</t>
+          <t>-0.36% (Yatay)</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>-0.85% (Azalış)</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>+15.05% (Artış)</t>
+          <t>+14.72% (Artış)</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>+27.56% (Artış)</t>
+          <t>+27.50% (Artış)</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -3112,7 +3225,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>603.25</v>
+        <v>603.5</v>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
@@ -3121,32 +3234,32 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>-0.08% (Yatay)</t>
+          <t>-0.04% (Yatay)</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>-3.48% (Azalış)</t>
+          <t>-3.44% (Azalış)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>-11.64% (Azalış)</t>
+          <t>-11.61% (Azalış)</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>-7.33% (Azalış)</t>
+          <t>-7.30% (Azalış)</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>+18.98% (Artış)</t>
+          <t>+19.03% (Artış)</t>
         </is>
       </c>
       <c r="K27" s="4" t="inlineStr">
         <is>
-          <t>+15.07% (Artış)</t>
+          <t>+13.01% (Artış)</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -3172,7 +3285,7 @@
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>287.15</v>
+        <v>287.2</v>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
@@ -3181,32 +3294,32 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>+0.60% (Artış)</t>
+          <t>+0.61% (Artış)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>-6.60% (Azalış)</t>
+          <t>-6.59% (Azalış)</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>-0.38% (Yatay)</t>
+          <t>-0.36% (Yatay)</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>-10.13% (Azalış)</t>
+          <t>-10.11% (Azalış)</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>-17.66% (Azalış)</t>
+          <t>-17.65% (Azalış)</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>-26.75% (Azalış)</t>
+          <t>-26.74% (Azalış)</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -3232,7 +3345,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>6240.12</v>
+        <v>6260.46</v>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3354,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>-3.38% (Azalış)</t>
+          <t>-3.07% (Azalış)</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -3292,7 +3405,7 @@
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>79.28</v>
+        <v>79.41</v>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
@@ -3301,17 +3414,17 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>+2.64% (Artış)</t>
+          <t>+2.81% (Artış)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>+6.24% (Artış)</t>
+          <t>+6.42% (Artış)</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>+14.57% (Artış)</t>
+          <t>+14.75% (Artış)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -3321,17 +3434,17 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>+28.08% (Artış)</t>
+          <t>+28.29% (Artış)</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
         <is>
-          <t>-4.40% (Azalış)</t>
+          <t>-4.64% (Azalış)</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Altın/Gümüş oranı 79.28 ile dengeli bantta seyrediyor.</t>
+          <t>Altın/Gümüş oranı 79.41 ile dengeli bantta seyrediyor.</t>
         </is>
       </c>
     </row>
@@ -3395,11 +3508,11 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>215.43</v>
+        <v>215.44</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TL: 10759.56 / Kur: 49.94</t>
+          <t>TL: 10759.6 / Kur: 49.94</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -3421,7 +3534,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>%-3.92</t>
+          <t>%-3.91</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -3448,7 +3561,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>%-4.52</t>
+          <t>%-4.51</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3607,7 +3720,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>215.43</v>
+        <v>215.44</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -3684,7 +3797,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>215.43</v>
+        <v>215.44</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -3759,7 +3872,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>260.51</v>
+        <v>260.52</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -3893,7 +4006,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>BIST 100 Dolar bazında 215.43$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.0) yer alıyor. 52 haftalık zirvesinden (333.44$) %35.4 aşağıda, 52 haftalık dibinden (215.43$) ise %0.0 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (294.86$) altında baskı altında seyrederken RSI(14) göstergesi 22.2 seviyesindedir.</t>
+          <t>BIST 100 Dolar bazında 215.44$ seviyesinde olup 1 yıllık dolar kanalının alt (ucuz/destek) bölgesinde (%0.0) yer alıyor. 52 haftalık zirvesinden (333.44$) %35.4 aşağıda, 52 haftalık dibinden (215.44$) ise %0.0 yukarıda bulunuyor. Endeks 200 günlük dolar ortalamasının (294.86$) altında baskı altında seyrederken RSI(14) göstergesi 22.2 seviyesindedir.</t>
         </is>
       </c>
     </row>
@@ -6021,7 +6134,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>24/100 (Aşırı Korku)</t>
+          <t>26/100 (Korku)</t>
         </is>
       </c>
     </row>
@@ -6043,7 +6156,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>21/100 (Aşırı Korku)</t>
+          <t>22/100 (Aşırı Korku)</t>
         </is>
       </c>
     </row>
@@ -6099,12 +6212,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Investing.com Türkiye</t>
+          <t>Gazete Oksijen</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Goldman, Çek Merkez Bankası faiz görüşünü enflasyon riskleri nedeniyle yükseltti</t>
+          <t>Üç büyük merkez bankası için kritik hafta: Enflasyon faiz kararlarını nasıl etkileyecek?</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -6121,12 +6234,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Gazete Oksijen</t>
+          <t>Investing.com Türkiye</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Üç büyük merkez bankası için kritik hafta: Enflasyon faiz kararlarını nasıl etkileyecek?</t>
+          <t>Goldman, Çek Merkez Bankası faiz görüşünü enflasyon riskleri nedeniyle yükseltti</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -6165,17 +6278,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>İstanbul Ticaret Gazetesi</t>
+          <t>Paratic Haber</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Kanada Merkez Bankası faiz kararını açıkladı: 2023’ten sonra ilk artış</t>
+          <t>Faiz indirimi sonrası TCMB’den kritik uyarı: Enflasyon yeniden yükselebilir</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Merkez Bankası, Faiz</t>
+          <t>TCMB, Faiz, Enflasyon</t>
         </is>
       </c>
     </row>
@@ -6187,17 +6300,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Euronews.com</t>
+          <t>İstanbul Ticaret Gazetesi</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Enflasyon ve petrol fiyatları Fed'in faiz kararını nasıl etkileyecek?</t>
+          <t>Kanada Merkez Bankası faiz kararını açıkladı: 2023’ten sonra ilk artış</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Fed, Faiz, Enflasyon</t>
+          <t>Merkez Bankası, Faiz</t>
         </is>
       </c>
     </row>
@@ -6253,12 +6366,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Ekonomim</t>
+          <t>CNBC-e</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Fitch'ten Türkiye tahmini: Borçlanma piyasasında büyüme beklentisi 550 milyar dolar</t>
+          <t>Fitch'ten Türkiye'nin borçlanma piyasasına ilişkin büyüme tahmini</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -6297,12 +6410,12 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Amida Haber</t>
+          <t>Haberler</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>TÜİK konut satış istatistiklerini açıkladı: Dikkat çekici düşüş</t>
+          <t>TÜİK verilerine göre Uşak'ta konut satışları Eylül'de 52 artarak 770'e yükseldi</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -6319,12 +6432,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Bloomberght</t>
+          <t>Olay Gazetesi Bursa</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Konut satışları Eylül'de yıllık düşüş serisini sürdürdü</t>
+          <t>Konut satış rakamları açıklandı - Olay Gazetesi Bursa</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">

</xml_diff>